<commit_message>
Updated all some reg_*.xlsx estimates corrected a few bugs in income, partnership processes; also updated RMSE accordingly.
</commit_message>
<xml_diff>
--- a/input/ES/reg_income.xlsx
+++ b/input/ES/reg_income.xlsx
@@ -448,7 +448,7 @@
         <v>19</v>
       </c>
       <c r="B13">
-        <v>0.54362013493723471</v>
+        <v>0.63405729156306156</v>
       </c>
       <c r="C13"/>
       <c r="D13"/>
@@ -459,7 +459,7 @@
         <v>17</v>
       </c>
       <c r="B14">
-        <v>52275</v>
+        <v>53223</v>
       </c>
       <c r="C14"/>
       <c r="D14"/>
@@ -4445,106 +4445,106 @@
         <v>28</v>
       </c>
       <c r="B2">
-        <v>-0.016530073157209738</v>
+        <v>-0.0099465674818788388</v>
       </c>
       <c r="C2">
-        <v>0.00033800478518149576</v>
+        <v>0.00024411009917686062</v>
       </c>
       <c r="D2">
-        <v>-1.1595262593671678e-06</v>
+        <v>-1.2664761897858985e-06</v>
       </c>
       <c r="E2">
-        <v>3.2797749563823646e-08</v>
+        <v>2.6287358297690028e-08</v>
       </c>
       <c r="F2">
-        <v>2.3514888390001136e-05</v>
+        <v>1.7601772434195182e-05</v>
       </c>
       <c r="G2">
-        <v>-2.1657825642411691e-05</v>
+        <v>-1.490817548300548e-05</v>
       </c>
       <c r="H2">
-        <v>-1.4229050579139729e-05</v>
+        <v>-2.8763485953285989e-06</v>
       </c>
       <c r="I2">
-        <v>-6.7355800366263385e-05</v>
+        <v>-4.6281657879378537e-05</v>
       </c>
       <c r="J2">
-        <v>4.159705099024866e-05</v>
+        <v>7.4873669564022607e-06</v>
       </c>
       <c r="K2">
-        <v>-2.1122839431273256e-05</v>
+        <v>-1.5208566547023861e-05</v>
       </c>
       <c r="L2">
-        <v>-7.1611176054830783e-07</v>
+        <v>-4.0111230732168969e-07</v>
       </c>
       <c r="M2">
-        <v>-3.2212234831237209e-05</v>
+        <v>-4.2896352715254841e-06</v>
       </c>
       <c r="N2">
-        <v>-0.00032709392055204717</v>
+        <v>-0.00024034260259612488</v>
       </c>
       <c r="O2">
-        <v>-5.2614115386368898e-05</v>
+        <v>-1.0223419842135619e-05</v>
       </c>
       <c r="P2">
-        <v>3.3549356567971337e-05</v>
+        <v>4.576667820430703e-06</v>
       </c>
       <c r="Q2">
-        <v>-0.00023316230487734562</v>
+        <v>-0.00018675253873414515</v>
       </c>
       <c r="R2">
-        <v>-0.00023008438428831932</v>
+        <v>-0.00018151597747181135</v>
       </c>
       <c r="S2">
-        <v>-0.00019367918701796553</v>
+        <v>-0.00015507529010086275</v>
       </c>
       <c r="T2">
-        <v>-0.0001027422881938953</v>
+        <v>-9.5660569266283366e-05</v>
       </c>
       <c r="U2">
-        <v>-5.2265305761841304e-05</v>
+        <v>-2.95200541884232e-05</v>
       </c>
       <c r="V2">
-        <v>-0.00020319985945792786</v>
+        <v>-0.00014176747662271859</v>
       </c>
       <c r="W2">
-        <v>4.0345429562238022e-05</v>
+        <v>2.9154778942572579e-05</v>
       </c>
       <c r="X2">
-        <v>-3.6891271348568258e-07</v>
+        <v>6.1134543296815869e-06</v>
       </c>
       <c r="Y2">
-        <v>0.00013694080783844886</v>
+        <v>0.00010297790051462028</v>
       </c>
       <c r="Z2">
-        <v>5.7425833494780031e-06</v>
+        <v>-9.335864421748392e-06</v>
       </c>
       <c r="AA2">
-        <v>1.0743021050413368e-05</v>
+        <v>-5.8546447618001047e-06</v>
       </c>
       <c r="AB2">
-        <v>6.9760191377979161e-06</v>
+        <v>-1.0585656419178065e-05</v>
       </c>
       <c r="AC2">
-        <v>4.37177101838762e-06</v>
+        <v>-8.7572897623118122e-06</v>
       </c>
       <c r="AD2">
-        <v>-1.8893322566322499e-05</v>
+        <v>-2.4432389547118601e-05</v>
       </c>
       <c r="AE2">
-        <v>9.078395632183029e-06</v>
+        <v>-4.4127055464639188e-06</v>
       </c>
       <c r="AF2">
-        <v>-1.1713617503157034e-07</v>
+        <v>-1.3817237429177379e-07</v>
       </c>
       <c r="AG2">
-        <v>-7.8348589206558112e-05</v>
+        <v>-4.6110191547671093e-05</v>
       </c>
       <c r="AH2">
-        <v>-2.871086252514396e-05</v>
+        <v>-1.7785141546052447e-05</v>
       </c>
       <c r="AI2">
-        <v>0.00017048838167084109</v>
+        <v>0.00015577358027267209</v>
       </c>
     </row>
     <row r="3">
@@ -4552,106 +4552,106 @@
         <v>29</v>
       </c>
       <c r="B3">
-        <v>0.016860101326262086</v>
+        <v>0.0080688654942652569</v>
       </c>
       <c r="C3">
-        <v>-1.1595262593671678e-06</v>
+        <v>-1.2664761897858985e-06</v>
       </c>
       <c r="D3">
-        <v>1.6420423126666384e-05</v>
+        <v>1.197965394310739e-05</v>
       </c>
       <c r="E3">
-        <v>-1.4365460726144509e-07</v>
+        <v>-1.0292787588158636e-07</v>
       </c>
       <c r="F3">
-        <v>-1.1131506836735371e-05</v>
+        <v>-4.8322411429239144e-06</v>
       </c>
       <c r="G3">
-        <v>-1.0449882433668442e-05</v>
+        <v>-4.5870197709802075e-06</v>
       </c>
       <c r="H3">
-        <v>-1.2208783486304137e-05</v>
+        <v>-7.855583864556253e-06</v>
       </c>
       <c r="I3">
-        <v>5.1034531149174217e-06</v>
+        <v>8.1667961682356852e-06</v>
       </c>
       <c r="J3">
-        <v>-4.4936032629895562e-06</v>
+        <v>-4.8127730407201622e-07</v>
       </c>
       <c r="K3">
-        <v>-2.9196896116809199e-06</v>
+        <v>-2.1040436555915697e-06</v>
       </c>
       <c r="L3">
-        <v>-6.6962297367110984e-07</v>
+        <v>-8.6176110047960581e-07</v>
       </c>
       <c r="M3">
-        <v>1.6047034429475957e-06</v>
+        <v>-3.8982039267731415e-07</v>
       </c>
       <c r="N3">
-        <v>1.587768351397972e-06</v>
+        <v>3.1532069630658345e-07</v>
       </c>
       <c r="O3">
-        <v>4.7129042874799443e-06</v>
+        <v>-7.4091149670805026e-08</v>
       </c>
       <c r="P3">
-        <v>-2.2156869189074688e-06</v>
+        <v>2.7184789103790458e-07</v>
       </c>
       <c r="Q3">
-        <v>-2.4718436714475417e-05</v>
+        <v>-2.0730517857023458e-05</v>
       </c>
       <c r="R3">
-        <v>-3.6741172482691127e-05</v>
+        <v>-2.9683770745107406e-05</v>
       </c>
       <c r="S3">
-        <v>-2.7618385373603016e-05</v>
+        <v>-2.1545048505077787e-05</v>
       </c>
       <c r="T3">
-        <v>5.6327917884880805e-05</v>
+        <v>4.1911041234563763e-05</v>
       </c>
       <c r="U3">
-        <v>-2.8715351058527014e-05</v>
+        <v>-2.4552717071218503e-05</v>
       </c>
       <c r="V3">
-        <v>-3.3873129909836963e-06</v>
+        <v>-8.3669400091756764e-06</v>
       </c>
       <c r="W3">
-        <v>8.9916027705526815e-06</v>
+        <v>1.0149484608886576e-05</v>
       </c>
       <c r="X3">
-        <v>3.4925405800941836e-05</v>
+        <v>2.6659730312490085e-05</v>
       </c>
       <c r="Y3">
-        <v>1.0265266595365681e-05</v>
+        <v>9.8901673089887138e-06</v>
       </c>
       <c r="Z3">
-        <v>-3.6890395435922214e-07</v>
+        <v>9.1350952081012903e-07</v>
       </c>
       <c r="AA3">
-        <v>2.7230093151540838e-06</v>
+        <v>3.6215784504039074e-06</v>
       </c>
       <c r="AB3">
-        <v>2.6496366877957415e-06</v>
+        <v>4.3609333452371355e-06</v>
       </c>
       <c r="AC3">
-        <v>3.3060123068474884e-06</v>
+        <v>3.6727555877707108e-06</v>
       </c>
       <c r="AD3">
-        <v>2.7000313798056935e-06</v>
+        <v>3.6196768917586006e-06</v>
       </c>
       <c r="AE3">
-        <v>-3.7432941115907417e-06</v>
+        <v>-4.014368705582283e-06</v>
       </c>
       <c r="AF3">
-        <v>-1.1073115482207998e-07</v>
+        <v>-1.3660476020046644e-07</v>
       </c>
       <c r="AG3">
-        <v>7.2371231071046956e-07</v>
+        <v>1.1014417681391481e-06</v>
       </c>
       <c r="AH3">
-        <v>-2.0665980981459645e-06</v>
+        <v>-1.6190327647853096e-07</v>
       </c>
       <c r="AI3">
-        <v>-0.00037840922310119454</v>
+        <v>-0.00027957227949393528</v>
       </c>
     </row>
     <row r="4">
@@ -4659,106 +4659,106 @@
         <v>30</v>
       </c>
       <c r="B4">
-        <v>-0.00013073152915414545</v>
+        <v>-7.1974103601231976e-05</v>
       </c>
       <c r="C4">
-        <v>3.2797749563823646e-08</v>
+        <v>2.6287358297690028e-08</v>
       </c>
       <c r="D4">
-        <v>-1.4365460726144509e-07</v>
+        <v>-1.0292787588158636e-07</v>
       </c>
       <c r="E4">
-        <v>1.3292996372632669e-09</v>
+        <v>9.3671921542464885e-10</v>
       </c>
       <c r="F4">
-        <v>1.3253998648093149e-07</v>
+        <v>5.4897828747911303e-08</v>
       </c>
       <c r="G4">
-        <v>1.187290474665369e-07</v>
+        <v>4.8509377529350295e-08</v>
       </c>
       <c r="H4">
-        <v>1.6448313864879601e-07</v>
+        <v>1.0103065565266212e-07</v>
       </c>
       <c r="I4">
-        <v>3.1527165226505297e-08</v>
+        <v>-2.2507369047811773e-08</v>
       </c>
       <c r="J4">
-        <v>3.932745064176556e-08</v>
+        <v>3.3314865379650852e-09</v>
       </c>
       <c r="K4">
-        <v>5.446914133081583e-09</v>
+        <v>2.6175745309641719e-09</v>
       </c>
       <c r="L4">
-        <v>8.5263708724293891e-09</v>
+        <v>9.4811688437675025e-09</v>
       </c>
       <c r="M4">
-        <v>-2.1576164477011495e-08</v>
+        <v>2.4439494548659494e-09</v>
       </c>
       <c r="N4">
-        <v>-3.4959148584785588e-08</v>
+        <v>-1.7725946010885246e-08</v>
       </c>
       <c r="O4">
-        <v>-3.8211111394579369e-08</v>
+        <v>2.2688116442150717e-09</v>
       </c>
       <c r="P4">
-        <v>2.4471266978375564e-08</v>
+        <v>-2.0261303533115006e-09</v>
       </c>
       <c r="Q4">
-        <v>1.5717468542467302e-07</v>
+        <v>1.345105398685577e-07</v>
       </c>
       <c r="R4">
-        <v>2.9121799219837417e-07</v>
+        <v>2.3201903387752886e-07</v>
       </c>
       <c r="S4">
-        <v>2.2981023190497959e-07</v>
+        <v>1.7713008708386214e-07</v>
       </c>
       <c r="T4">
-        <v>-5.3255137979159031e-07</v>
+        <v>-3.9850582766799807e-07</v>
       </c>
       <c r="U4">
-        <v>9.3323005600879071e-08</v>
+        <v>8.5366265271832758e-08</v>
       </c>
       <c r="V4">
-        <v>-3.0831760440807579e-07</v>
+        <v>-1.8236208065779914e-07</v>
       </c>
       <c r="W4">
-        <v>-2.5385119997845615e-08</v>
+        <v>-4.687240301874925e-08</v>
       </c>
       <c r="X4">
-        <v>-2.8087293733730018e-07</v>
+        <v>-2.0757740691395408e-07</v>
       </c>
       <c r="Y4">
-        <v>-1.8130713169339472e-08</v>
+        <v>-3.7547868734137601e-08</v>
       </c>
       <c r="Z4">
-        <v>-5.5115163241112756e-09</v>
+        <v>-3.6069770294001315e-08</v>
       </c>
       <c r="AA4">
-        <v>-4.0942454040429362e-08</v>
+        <v>-6.8712749839840212e-08</v>
       </c>
       <c r="AB4">
-        <v>-3.9895281830393476e-08</v>
+        <v>-7.3442178562350164e-08</v>
       </c>
       <c r="AC4">
-        <v>-4.6005625474448603e-08</v>
+        <v>-6.6999920756369802e-08</v>
       </c>
       <c r="AD4">
-        <v>-3.3621964339694341e-08</v>
+        <v>-6.1898072402069532e-08</v>
       </c>
       <c r="AE4">
-        <v>1.8196754478072829e-08</v>
+        <v>-8.3402859556666785e-10</v>
       </c>
       <c r="AF4">
-        <v>-7.6469376919826121e-10</v>
+        <v>-9.5757793863241551e-11</v>
       </c>
       <c r="AG4">
-        <v>-2.1061352079788054e-08</v>
+        <v>-2.3560282270735233e-08</v>
       </c>
       <c r="AH4">
-        <v>9.6154898530007683e-09</v>
+        <v>-9.8789553017018076e-09</v>
       </c>
       <c r="AI4">
-        <v>3.2688604033339336e-06</v>
+        <v>2.4101841408793162e-06</v>
       </c>
     </row>
     <row r="5">
@@ -4766,106 +4766,106 @@
         <v>32</v>
       </c>
       <c r="B5">
-        <v>0.03569393055445818</v>
+        <v>0.016990081193109886</v>
       </c>
       <c r="C5">
-        <v>2.3514888390001136e-05</v>
+        <v>1.7601772434195182e-05</v>
       </c>
       <c r="D5">
-        <v>-1.1131506836735371e-05</v>
+        <v>-4.8322411429239144e-06</v>
       </c>
       <c r="E5">
-        <v>1.3253998648093149e-07</v>
+        <v>5.4897828747911303e-08</v>
       </c>
       <c r="F5">
-        <v>0.004318747431300919</v>
+        <v>0.0032753876282476087</v>
       </c>
       <c r="G5">
-        <v>0.0033302585050640609</v>
+        <v>0.0025060621319671411</v>
       </c>
       <c r="H5">
-        <v>0.0033491861273780496</v>
+        <v>0.0025183613321627194</v>
       </c>
       <c r="I5">
-        <v>0.0033330570069508318</v>
+        <v>0.0025078561469495286</v>
       </c>
       <c r="J5">
-        <v>5.5261577523229785e-06</v>
+        <v>1.0441632202006488e-05</v>
       </c>
       <c r="K5">
-        <v>1.9946374018930971e-05</v>
+        <v>1.2780744562305172e-05</v>
       </c>
       <c r="L5">
-        <v>-5.5644572274199299e-06</v>
+        <v>-4.1921918042736863e-06</v>
       </c>
       <c r="M5">
-        <v>-6.8724727429687058e-05</v>
+        <v>-1.6654925238770426e-05</v>
       </c>
       <c r="N5">
-        <v>-2.221052676966873e-05</v>
+        <v>-1.7393331160956826e-05</v>
       </c>
       <c r="O5">
-        <v>-2.6264729022641535e-06</v>
+        <v>-1.0381919715457988e-05</v>
       </c>
       <c r="P5">
-        <v>6.2568237371362192e-05</v>
+        <v>1.5451374548412723e-05</v>
       </c>
       <c r="Q5">
-        <v>3.4086789976513036e-05</v>
+        <v>-1.6462071217785649e-05</v>
       </c>
       <c r="R5">
-        <v>9.2686772673516125e-05</v>
+        <v>2.7511439242178248e-05</v>
       </c>
       <c r="S5">
-        <v>7.234623004049234e-05</v>
+        <v>1.4456196281646683e-05</v>
       </c>
       <c r="T5">
-        <v>0.00010735315558156209</v>
+        <v>7.2319497612602108e-05</v>
       </c>
       <c r="U5">
-        <v>0.00013435923948253528</v>
+        <v>8.6116183005344616e-05</v>
       </c>
       <c r="V5">
-        <v>3.649228354062322e-05</v>
+        <v>3.9381120078241195e-05</v>
       </c>
       <c r="W5">
-        <v>1.396123948230936e-06</v>
+        <v>-2.3705830900374821e-05</v>
       </c>
       <c r="X5">
-        <v>-1.148587195645874e-05</v>
+        <v>-3.3536093379019387e-05</v>
       </c>
       <c r="Y5">
-        <v>5.9715548943519012e-05</v>
+        <v>3.1718669050096599e-05</v>
       </c>
       <c r="Z5">
-        <v>-5.6077131279566074e-05</v>
+        <v>-5.1834310924630395e-05</v>
       </c>
       <c r="AA5">
-        <v>-3.2613800962478764e-05</v>
+        <v>-3.7256828155836277e-05</v>
       </c>
       <c r="AB5">
-        <v>-4.3719027208413697e-05</v>
+        <v>-4.3119877050201987e-05</v>
       </c>
       <c r="AC5">
-        <v>-9.434248749252863e-05</v>
+        <v>-7.7778989518010634e-05</v>
       </c>
       <c r="AD5">
-        <v>1.0024030448895545e-05</v>
+        <v>-1.8384535306178919e-06</v>
       </c>
       <c r="AE5">
-        <v>-5.3170062463804915e-06</v>
+        <v>-1.8419200261227565e-05</v>
       </c>
       <c r="AF5">
-        <v>-2.1296604221588067e-06</v>
+        <v>-1.2536112130698041e-07</v>
       </c>
       <c r="AG5">
-        <v>1.3101660560370029e-05</v>
+        <v>-1.6968138335860146e-05</v>
       </c>
       <c r="AH5">
-        <v>-1.1459651114999712e-06</v>
+        <v>-3.163277299217046e-06</v>
       </c>
       <c r="AI5">
-        <v>-0.0031907660066190684</v>
+        <v>-0.0024347903066560409</v>
       </c>
     </row>
     <row r="6">
@@ -4873,106 +4873,106 @@
         <v>33</v>
       </c>
       <c r="B6">
-        <v>0.075534146507023808</v>
+        <v>0.023034392710275145</v>
       </c>
       <c r="C6">
-        <v>-2.1657825642411691e-05</v>
+        <v>-1.490817548300548e-05</v>
       </c>
       <c r="D6">
-        <v>-1.0449882433668442e-05</v>
+        <v>-4.5870197709802075e-06</v>
       </c>
       <c r="E6">
-        <v>1.187290474665369e-07</v>
+        <v>4.8509377529350295e-08</v>
       </c>
       <c r="F6">
-        <v>0.0033302585050640609</v>
+        <v>0.0025060621319671411</v>
       </c>
       <c r="G6">
-        <v>0.0036905918227806895</v>
+        <v>0.0027737642581545921</v>
       </c>
       <c r="H6">
-        <v>0.0034448815958518669</v>
+        <v>0.0025800678806974053</v>
       </c>
       <c r="I6">
-        <v>0.003444307874982767</v>
+        <v>0.0025837486740412129</v>
       </c>
       <c r="J6">
-        <v>-3.7918598515992476e-05</v>
+        <v>-8.3244767404608939e-06</v>
       </c>
       <c r="K6">
-        <v>1.6091835103031221e-05</v>
+        <v>1.2346989523060137e-05</v>
       </c>
       <c r="L6">
-        <v>-6.328648311897491e-06</v>
+        <v>-4.5552460465075425e-06</v>
       </c>
       <c r="M6">
-        <v>-2.4333501048798886e-05</v>
+        <v>2.6813406474502808e-07</v>
       </c>
       <c r="N6">
-        <v>1.2426357628698525e-05</v>
+        <v>9.3865545268970109e-06</v>
       </c>
       <c r="O6">
-        <v>2.7402438157772373e-05</v>
+        <v>5.0526528036755011e-06</v>
       </c>
       <c r="P6">
-        <v>3.0600985372090765e-05</v>
+        <v>1.6942264189230539e-06</v>
       </c>
       <c r="Q6">
-        <v>0.00011215392557799037</v>
+        <v>5.0933515410422209e-05</v>
       </c>
       <c r="R6">
-        <v>0.00010674103557494451</v>
+        <v>4.1964274798717439e-05</v>
       </c>
       <c r="S6">
-        <v>0.00010523337934325834</v>
+        <v>4.6691616419018874e-05</v>
       </c>
       <c r="T6">
-        <v>6.506798789906185e-05</v>
+        <v>6.1135750738960503e-05</v>
       </c>
       <c r="U6">
-        <v>0.00011380341857671148</v>
+        <v>9.7678731807014207e-05</v>
       </c>
       <c r="V6">
-        <v>6.7121795603022763e-05</v>
+        <v>8.3261361007281199e-05</v>
       </c>
       <c r="W6">
-        <v>3.240480365034445e-05</v>
+        <v>9.8725724469550351e-06</v>
       </c>
       <c r="X6">
-        <v>3.6184796380715366e-05</v>
+        <v>1.1602479155745776e-05</v>
       </c>
       <c r="Y6">
-        <v>0.00011715946216607118</v>
+        <v>8.6282675976143792e-05</v>
       </c>
       <c r="Z6">
-        <v>-3.2391368146266614e-05</v>
+        <v>-2.3694207330035404e-05</v>
       </c>
       <c r="AA6">
-        <v>-3.342869865768038e-05</v>
+        <v>-2.6420656955067042e-05</v>
       </c>
       <c r="AB6">
-        <v>-3.4709028774606351e-05</v>
+        <v>-2.4660131683162771e-05</v>
       </c>
       <c r="AC6">
-        <v>-9.5431062887091789e-05</v>
+        <v>-7.3953676822698881e-05</v>
       </c>
       <c r="AD6">
-        <v>-4.4670324184873517e-07</v>
+        <v>-1.3619129778063492e-05</v>
       </c>
       <c r="AE6">
-        <v>1.5892475574857154e-06</v>
+        <v>-4.6261090988816548e-06</v>
       </c>
       <c r="AF6">
-        <v>-4.9904075742537298e-06</v>
+        <v>-2.8987659844247721e-06</v>
       </c>
       <c r="AG6">
-        <v>2.3560435616849611e-05</v>
+        <v>2.3488971895614663e-06</v>
       </c>
       <c r="AH6">
-        <v>5.04504162779848e-05</v>
+        <v>5.6548310784992374e-05</v>
       </c>
       <c r="AI6">
-        <v>-0.003264930078864586</v>
+        <v>-0.0025068716653706587</v>
       </c>
     </row>
     <row r="7">
@@ -4980,106 +4980,106 @@
         <v>34</v>
       </c>
       <c r="B7">
-        <v>0.099579576065623399</v>
+        <v>0.044455828266261953</v>
       </c>
       <c r="C7">
-        <v>-1.4229050579139729e-05</v>
+        <v>-2.8763485953285989e-06</v>
       </c>
       <c r="D7">
-        <v>-1.2208783486304137e-05</v>
+        <v>-7.855583864556253e-06</v>
       </c>
       <c r="E7">
-        <v>1.6448313864879601e-07</v>
+        <v>1.0103065565266212e-07</v>
       </c>
       <c r="F7">
-        <v>0.0033491861273780496</v>
+        <v>0.0025183613321627194</v>
       </c>
       <c r="G7">
-        <v>0.0034448815958518669</v>
+        <v>0.0025800678806974053</v>
       </c>
       <c r="H7">
-        <v>0.0036636700724075187</v>
+        <v>0.002737060003854637</v>
       </c>
       <c r="I7">
-        <v>0.0035773197663790421</v>
+        <v>0.0026671012710242741</v>
       </c>
       <c r="J7">
-        <v>-4.4606874437227474e-05</v>
+        <v>-1.5508708249053821e-05</v>
       </c>
       <c r="K7">
-        <v>1.3292267483377781e-05</v>
+        <v>6.2938293980314443e-06</v>
       </c>
       <c r="L7">
-        <v>-4.6114483418551445e-06</v>
+        <v>-2.4100736421399857e-06</v>
       </c>
       <c r="M7">
-        <v>-5.4849531344481478e-06</v>
+        <v>7.655752822538595e-06</v>
       </c>
       <c r="N7">
-        <v>1.6768692062677903e-05</v>
+        <v>4.2859539845740394e-06</v>
       </c>
       <c r="O7">
-        <v>5.8139325118979502e-05</v>
+        <v>2.0651020696011693e-05</v>
       </c>
       <c r="P7">
-        <v>-6.8756435468558244e-06</v>
+        <v>-1.0737971898872799e-05</v>
       </c>
       <c r="Q7">
-        <v>0.00012172266110459327</v>
+        <v>6.7345411768237901e-05</v>
       </c>
       <c r="R7">
-        <v>9.4734495009401488e-05</v>
+        <v>4.35244828016065e-05</v>
       </c>
       <c r="S7">
-        <v>7.388652170449081e-05</v>
+        <v>3.690571616251628e-05</v>
       </c>
       <c r="T7">
-        <v>6.3292858309631217e-05</v>
+        <v>1.7097488510219461e-05</v>
       </c>
       <c r="U7">
-        <v>0.00014956025952320585</v>
+        <v>9.7737619638381271e-05</v>
       </c>
       <c r="V7">
-        <v>6.0869248048411742e-05</v>
+        <v>3.8233718438623193e-05</v>
       </c>
       <c r="W7">
-        <v>1.4386862176733667e-05</v>
+        <v>-8.5563527611985386e-06</v>
       </c>
       <c r="X7">
-        <v>2.9644530535361414e-05</v>
+        <v>6.5853044540289691e-06</v>
       </c>
       <c r="Y7">
-        <v>0.00014344774122373918</v>
+        <v>9.836435578030071e-05</v>
       </c>
       <c r="Z7">
-        <v>-7.1874354112027878e-05</v>
+        <v>-7.6247231313643794e-05</v>
       </c>
       <c r="AA7">
-        <v>-8.9556933801142932e-05</v>
+        <v>-9.1057264796521155e-05</v>
       </c>
       <c r="AB7">
-        <v>-9.6477235923793717e-05</v>
+        <v>-9.1372038908214153e-05</v>
       </c>
       <c r="AC7">
-        <v>-0.00014693418837219137</v>
+        <v>-0.00013429476518331436</v>
       </c>
       <c r="AD7">
-        <v>-5.8249228400782897e-05</v>
+        <v>-6.8257765771505079e-05</v>
       </c>
       <c r="AE7">
-        <v>-4.207361399925628e-05</v>
+        <v>-4.7055995359580351e-05</v>
       </c>
       <c r="AF7">
-        <v>-3.8069441577882174e-06</v>
+        <v>-2.1202340239441037e-06</v>
       </c>
       <c r="AG7">
-        <v>-1.3115123110637311e-06</v>
+        <v>-2.752301032101466e-05</v>
       </c>
       <c r="AH7">
-        <v>1.1186649182695282e-05</v>
+        <v>6.1610761025077295e-06</v>
       </c>
       <c r="AI7">
-        <v>-0.0033820336201729473</v>
+        <v>-0.0024907840804877122</v>
       </c>
     </row>
     <row r="8">
@@ -5087,106 +5087,106 @@
         <v>63</v>
       </c>
       <c r="B8">
-        <v>0.10191902942700919</v>
+        <v>0.04749721078508385</v>
       </c>
       <c r="C8">
-        <v>-6.7355800366263385e-05</v>
+        <v>-4.6281657879378537e-05</v>
       </c>
       <c r="D8">
-        <v>5.1034531149174217e-06</v>
+        <v>8.1667961682356852e-06</v>
       </c>
       <c r="E8">
-        <v>3.1527165226505297e-08</v>
+        <v>-2.2507369047811773e-08</v>
       </c>
       <c r="F8">
-        <v>0.0033330570069508318</v>
+        <v>0.0025078561469495286</v>
       </c>
       <c r="G8">
-        <v>0.003444307874982767</v>
+        <v>0.0025837486740412129</v>
       </c>
       <c r="H8">
-        <v>0.0035773197663790421</v>
+        <v>0.0026671012710242741</v>
       </c>
       <c r="I8">
-        <v>0.0041372324445851458</v>
+        <v>0.0031113251052543884</v>
       </c>
       <c r="J8">
-        <v>-0.00015795130210541613</v>
+        <v>-4.0007141896878035e-05</v>
       </c>
       <c r="K8">
-        <v>5.6290379254348058e-06</v>
+        <v>1.1836322680258097e-06</v>
       </c>
       <c r="L8">
-        <v>-1.7160491198794399e-05</v>
+        <v>-1.0576376631313277e-05</v>
       </c>
       <c r="M8">
-        <v>8.2831097415042186e-05</v>
+        <v>2.3057124559346988e-05</v>
       </c>
       <c r="N8">
-        <v>6.1195803712241507e-05</v>
+        <v>4.1849089375644254e-05</v>
       </c>
       <c r="O8">
-        <v>0.00019333505088077983</v>
+        <v>3.8196819185115681e-05</v>
       </c>
       <c r="P8">
-        <v>-0.00010390538640871693</v>
+        <v>-2.4508959900644691e-05</v>
       </c>
       <c r="Q8">
-        <v>0.0002252244350126123</v>
+        <v>0.00013209345152957091</v>
       </c>
       <c r="R8">
-        <v>0.00022811049602714829</v>
+        <v>0.00012728769464689796</v>
       </c>
       <c r="S8">
-        <v>0.00013170444398262395</v>
+        <v>6.5374092568053471e-05</v>
       </c>
       <c r="T8">
-        <v>-0.00013543921931975181</v>
+        <v>-8.2717081325280224e-05</v>
       </c>
       <c r="U8">
-        <v>-6.0851686910935905e-05</v>
+        <v>-5.4794783141643485e-05</v>
       </c>
       <c r="V8">
-        <v>-0.00012846647571950452</v>
+        <v>-9.1353798657312774e-05</v>
       </c>
       <c r="W8">
-        <v>2.8852205235416919e-06</v>
+        <v>-1.1666824654228198e-05</v>
       </c>
       <c r="X8">
-        <v>7.5507397100281742e-05</v>
+        <v>4.6188312691185078e-05</v>
       </c>
       <c r="Y8">
-        <v>0.00013852717240664609</v>
+        <v>0.00010371067588002786</v>
       </c>
       <c r="Z8">
-        <v>-6.0315393916438552e-06</v>
+        <v>1.1164296909034824e-05</v>
       </c>
       <c r="AA8">
-        <v>-5.561515106820218e-05</v>
+        <v>-2.9495735676815082e-05</v>
       </c>
       <c r="AB8">
-        <v>-7.6338942696981579e-05</v>
+        <v>-4.0220255936107693e-05</v>
       </c>
       <c r="AC8">
-        <v>-9.1646211952361393e-05</v>
+        <v>-5.789279880685479e-05</v>
       </c>
       <c r="AD8">
-        <v>4.7353825128320683e-05</v>
+        <v>4.768166417012964e-05</v>
       </c>
       <c r="AE8">
-        <v>-1.1162008556380321e-05</v>
+        <v>6.7545297397632689e-06</v>
       </c>
       <c r="AF8">
-        <v>-1.5413697275998045e-06</v>
+        <v>-2.5183170442093184e-07</v>
       </c>
       <c r="AG8">
-        <v>0.00017685683753167463</v>
+        <v>9.3093959670792308e-05</v>
       </c>
       <c r="AH8">
-        <v>6.4684847934265953e-05</v>
+        <v>3.5675842478548499e-05</v>
       </c>
       <c r="AI8">
-        <v>-0.0039016022318896365</v>
+        <v>-0.0029982245594123175</v>
       </c>
     </row>
     <row r="9">
@@ -5194,106 +5194,106 @@
         <v>64</v>
       </c>
       <c r="B9">
-        <v>1.5180195216091639</v>
+        <v>0.6248277955240169</v>
       </c>
       <c r="C9">
-        <v>4.159705099024866e-05</v>
+        <v>7.4873669564022607e-06</v>
       </c>
       <c r="D9">
-        <v>-4.4936032629895562e-06</v>
+        <v>-4.8127730407201622e-07</v>
       </c>
       <c r="E9">
-        <v>3.932745064176556e-08</v>
+        <v>3.3314865379650852e-09</v>
       </c>
       <c r="F9">
-        <v>5.5261577523229785e-06</v>
+        <v>1.0441632202006488e-05</v>
       </c>
       <c r="G9">
-        <v>-3.7918598515992476e-05</v>
+        <v>-8.3244767404608939e-06</v>
       </c>
       <c r="H9">
-        <v>-4.4606874437227474e-05</v>
+        <v>-1.5508708249053821e-05</v>
       </c>
       <c r="I9">
-        <v>-0.00015795130210541613</v>
+        <v>-4.0007141896878035e-05</v>
       </c>
       <c r="J9">
-        <v>0.00064178782738026142</v>
+        <v>7.7042335273389833e-05</v>
       </c>
       <c r="K9">
-        <v>-2.3086048402090315e-05</v>
+        <v>-2.4442730153099527e-06</v>
       </c>
       <c r="L9">
-        <v>7.3811694050690362e-06</v>
+        <v>-1.2438598104645486e-06</v>
       </c>
       <c r="M9">
-        <v>-0.00045982538474761628</v>
+        <v>-6.5096680805900128e-05</v>
       </c>
       <c r="N9">
-        <v>-2.3347955927411466e-05</v>
+        <v>-3.122888310336402e-06</v>
       </c>
       <c r="O9">
-        <v>-0.00063916565257824678</v>
+        <v>-7.5920632807978535e-05</v>
       </c>
       <c r="P9">
-        <v>0.00043986487685248341</v>
+        <v>6.3305209309768443e-05</v>
       </c>
       <c r="Q9">
-        <v>-0.00028121560836039735</v>
+        <v>-4.53730621217587e-05</v>
       </c>
       <c r="R9">
-        <v>-0.00028120091219737076</v>
+        <v>-4.4683056230358801e-05</v>
       </c>
       <c r="S9">
-        <v>-0.00024159070326182217</v>
+        <v>-4.337675529428107e-05</v>
       </c>
       <c r="T9">
-        <v>-5.9662954073992389e-05</v>
+        <v>-1.2158462172536947e-05</v>
       </c>
       <c r="U9">
-        <v>-9.3223257890432193e-05</v>
+        <v>-2.7260263517076077e-05</v>
       </c>
       <c r="V9">
-        <v>-0.00012104402601295762</v>
+        <v>-2.7004610335824979e-05</v>
       </c>
       <c r="W9">
-        <v>2.2253769112660799e-05</v>
+        <v>2.7620788434536656e-06</v>
       </c>
       <c r="X9">
-        <v>-5.9665466520087527e-05</v>
+        <v>-1.8224339906499334e-05</v>
       </c>
       <c r="Y9">
-        <v>-5.816469041652558e-05</v>
+        <v>-2.1306315218930899e-05</v>
       </c>
       <c r="Z9">
-        <v>8.5149803357657992e-06</v>
+        <v>7.2757498058676063e-06</v>
       </c>
       <c r="AA9">
-        <v>7.7232169495954248e-06</v>
+        <v>6.9017503300158681e-06</v>
       </c>
       <c r="AB9">
-        <v>-9.9065126713600744e-06</v>
+        <v>2.632259753434833e-06</v>
       </c>
       <c r="AC9">
-        <v>9.5318444476418823e-06</v>
+        <v>8.3152163847382398e-06</v>
       </c>
       <c r="AD9">
-        <v>-7.4128590388704578e-05</v>
+        <v>-9.1512358603782229e-06</v>
       </c>
       <c r="AE9">
-        <v>-3.4362991330363968e-06</v>
+        <v>8.0240392261744832e-06</v>
       </c>
       <c r="AF9">
-        <v>-1.2655894037201618e-06</v>
+        <v>-6.6831626087156612e-07</v>
       </c>
       <c r="AG9">
-        <v>-0.00016898574867744656</v>
+        <v>-3.0264472768573137e-05</v>
       </c>
       <c r="AH9">
-        <v>-8.3200465864430545e-05</v>
+        <v>-2.1851970220350368e-05</v>
       </c>
       <c r="AI9">
-        <v>0.00037411143719150966</v>
+        <v>8.019374920288896e-05</v>
       </c>
     </row>
     <row r="10">
@@ -5301,106 +5301,106 @@
         <v>36</v>
       </c>
       <c r="B10">
-        <v>0.019864871028473223</v>
+        <v>0.021324138692213734</v>
       </c>
       <c r="C10">
-        <v>-2.1122839431273256e-05</v>
+        <v>-1.5208566547023861e-05</v>
       </c>
       <c r="D10">
-        <v>-2.9196896116809199e-06</v>
+        <v>-2.1040436555915697e-06</v>
       </c>
       <c r="E10">
-        <v>5.446914133081583e-09</v>
+        <v>2.6175745309641719e-09</v>
       </c>
       <c r="F10">
-        <v>1.9946374018930971e-05</v>
+        <v>1.2780744562305172e-05</v>
       </c>
       <c r="G10">
-        <v>1.6091835103031221e-05</v>
+        <v>1.2346989523060137e-05</v>
       </c>
       <c r="H10">
-        <v>1.3292267483377781e-05</v>
+        <v>6.2938293980314443e-06</v>
       </c>
       <c r="I10">
-        <v>5.6290379254348058e-06</v>
+        <v>1.1836322680258097e-06</v>
       </c>
       <c r="J10">
-        <v>-2.3086048402090315e-05</v>
+        <v>-2.4442730153099527e-06</v>
       </c>
       <c r="K10">
-        <v>0.00033512445474611854</v>
+        <v>0.0002541622921735693</v>
       </c>
       <c r="L10">
-        <v>-2.5254455305878726e-05</v>
+        <v>-2.0429203728817576e-05</v>
       </c>
       <c r="M10">
-        <v>1.0395485362990614e-05</v>
+        <v>-1.3639714086494223e-06</v>
       </c>
       <c r="N10">
-        <v>1.7986021986654278e-05</v>
+        <v>1.3463637768981388e-05</v>
       </c>
       <c r="O10">
-        <v>2.3619129366459282e-05</v>
+        <v>2.7466930257796166e-06</v>
       </c>
       <c r="P10">
-        <v>-9.4033853972996361e-06</v>
+        <v>1.2614631502436618e-06</v>
       </c>
       <c r="Q10">
-        <v>0.00011245365347632881</v>
+        <v>8.8838302483919577e-05</v>
       </c>
       <c r="R10">
-        <v>8.4701074168258951e-05</v>
+        <v>6.2896581643416809e-05</v>
       </c>
       <c r="S10">
-        <v>1.2075251853831039e-05</v>
+        <v>9.5007338137436705e-06</v>
       </c>
       <c r="T10">
-        <v>0.0024972211811194393</v>
+        <v>0.0018872080951591495</v>
       </c>
       <c r="U10">
-        <v>0.0025423143104802422</v>
+        <v>0.0019220082482929528</v>
       </c>
       <c r="V10">
-        <v>0.002568404299279205</v>
+        <v>0.0019437705410297766</v>
       </c>
       <c r="W10">
-        <v>-2.8229001594775981e-05</v>
+        <v>-1.9221651197954986e-05</v>
       </c>
       <c r="X10">
-        <v>2.2909570554582198e-06</v>
+        <v>7.4496682716483891e-06</v>
       </c>
       <c r="Y10">
-        <v>4.6191887562013366e-05</v>
+        <v>5.5120278635650984e-05</v>
       </c>
       <c r="Z10">
-        <v>9.418187349832124e-06</v>
+        <v>2.1383848145603915e-05</v>
       </c>
       <c r="AA10">
-        <v>-1.9276415664130865e-05</v>
+        <v>4.0595445390421633e-06</v>
       </c>
       <c r="AB10">
-        <v>-2.7012175418189175e-05</v>
+        <v>-2.5227767774379725e-06</v>
       </c>
       <c r="AC10">
-        <v>7.8577577430050637e-06</v>
+        <v>2.1739266659929926e-05</v>
       </c>
       <c r="AD10">
-        <v>-1.7723351807230679e-05</v>
+        <v>2.4285883841762448e-06</v>
       </c>
       <c r="AE10">
-        <v>1.1960281701943796e-05</v>
+        <v>1.3038864400544787e-05</v>
       </c>
       <c r="AF10">
-        <v>8.2590497641914012e-07</v>
+        <v>8.397996004587753e-07</v>
       </c>
       <c r="AG10">
-        <v>1.6152553236027049e-05</v>
+        <v>8.9231783656214085e-06</v>
       </c>
       <c r="AH10">
-        <v>3.0176125816626896e-05</v>
+        <v>9.3125405626924085e-06</v>
       </c>
       <c r="AI10">
-        <v>-0.0024598768867113464</v>
+        <v>-0.00187831800198429</v>
       </c>
     </row>
     <row r="11">
@@ -5408,106 +5408,106 @@
         <v>37</v>
       </c>
       <c r="B11">
-        <v>0.0067999473075663905</v>
+        <v>0.0074296143127429177</v>
       </c>
       <c r="C11">
-        <v>-7.1611176054830783e-07</v>
+        <v>-4.0111230732168969e-07</v>
       </c>
       <c r="D11">
-        <v>-6.6962297367110984e-07</v>
+        <v>-8.6176110047960581e-07</v>
       </c>
       <c r="E11">
-        <v>8.5263708724293891e-09</v>
+        <v>9.4811688437675025e-09</v>
       </c>
       <c r="F11">
-        <v>-5.5644572274199299e-06</v>
+        <v>-4.1921918042736863e-06</v>
       </c>
       <c r="G11">
-        <v>-6.328648311897491e-06</v>
+        <v>-4.5552460465075425e-06</v>
       </c>
       <c r="H11">
-        <v>-4.6114483418551445e-06</v>
+        <v>-2.4100736421399857e-06</v>
       </c>
       <c r="I11">
-        <v>-1.7160491198794399e-05</v>
+        <v>-1.0576376631313277e-05</v>
       </c>
       <c r="J11">
-        <v>7.3811694050690362e-06</v>
+        <v>-1.2438598104645486e-06</v>
       </c>
       <c r="K11">
-        <v>-2.5254455305878726e-05</v>
+        <v>-2.0429203728817576e-05</v>
       </c>
       <c r="L11">
-        <v>2.1754716653805837e-05</v>
+        <v>1.7527365325024938e-05</v>
       </c>
       <c r="M11">
-        <v>-4.0715320172183104e-06</v>
+        <v>2.2714633045317487e-06</v>
       </c>
       <c r="N11">
-        <v>8.4221969913879455e-07</v>
+        <v>5.0481052890735936e-07</v>
       </c>
       <c r="O11">
-        <v>-8.418638274399032e-06</v>
+        <v>1.094630901900406e-06</v>
       </c>
       <c r="P11">
-        <v>4.6374156606388902e-06</v>
+        <v>-2.1465462890232318e-06</v>
       </c>
       <c r="Q11">
-        <v>-8.4233950044148215e-06</v>
+        <v>-5.2446072122630411e-06</v>
       </c>
       <c r="R11">
-        <v>-2.4807567488618741e-05</v>
+        <v>-1.8481287009426216e-05</v>
       </c>
       <c r="S11">
-        <v>-1.1985930145395562e-05</v>
+        <v>-6.0486556435260163e-06</v>
       </c>
       <c r="T11">
-        <v>-4.933522852928612e-05</v>
+        <v>-4.1690923457297036e-05</v>
       </c>
       <c r="U11">
-        <v>-6.637102713381732e-05</v>
+        <v>-4.9678699126256522e-05</v>
       </c>
       <c r="V11">
-        <v>-5.8997845047084071e-05</v>
+        <v>-4.723236331971339e-05</v>
       </c>
       <c r="W11">
-        <v>2.1549592304919692e-07</v>
+        <v>9.2883273672897568e-09</v>
       </c>
       <c r="X11">
-        <v>2.8208978696641841e-06</v>
+        <v>3.5352631715359018e-06</v>
       </c>
       <c r="Y11">
-        <v>8.6033118555267458e-06</v>
+        <v>3.9968723023051736e-06</v>
       </c>
       <c r="Z11">
-        <v>-5.8983953549960456e-06</v>
+        <v>-9.6109704479998775e-06</v>
       </c>
       <c r="AA11">
-        <v>-8.370704189693698e-06</v>
+        <v>-1.1695178700563376e-05</v>
       </c>
       <c r="AB11">
-        <v>-4.4093195581566065e-06</v>
+        <v>-8.7266002255603918e-06</v>
       </c>
       <c r="AC11">
-        <v>-7.1575627419663402e-06</v>
+        <v>-1.0450915284128772e-05</v>
       </c>
       <c r="AD11">
-        <v>-1.0905681299324917e-05</v>
+        <v>-1.2277464137015223e-05</v>
       </c>
       <c r="AE11">
-        <v>-5.2561162497527967e-06</v>
+        <v>-9.1444009299757552e-06</v>
       </c>
       <c r="AF11">
-        <v>-2.708817252856624e-07</v>
+        <v>-1.7756947047362303e-07</v>
       </c>
       <c r="AG11">
-        <v>-5.157916866126524e-06</v>
+        <v>2.7865441998081248e-06</v>
       </c>
       <c r="AH11">
-        <v>-7.1369518895646625e-06</v>
+        <v>-4.8713737517581206e-06</v>
       </c>
       <c r="AI11">
-        <v>8.0841463138480685e-05</v>
+        <v>7.2341622901808439e-05</v>
       </c>
     </row>
     <row r="12">
@@ -5515,106 +5515,106 @@
         <v>65</v>
       </c>
       <c r="B12">
-        <v>0.6531478238810513</v>
+        <v>0.23595020672705081</v>
       </c>
       <c r="C12">
-        <v>-3.2212234831237209e-05</v>
+        <v>-4.2896352715254841e-06</v>
       </c>
       <c r="D12">
-        <v>1.6047034429475957e-06</v>
+        <v>-3.8982039267731415e-07</v>
       </c>
       <c r="E12">
-        <v>-2.1576164477011495e-08</v>
+        <v>2.4439494548659494e-09</v>
       </c>
       <c r="F12">
-        <v>-6.8724727429687058e-05</v>
+        <v>-1.6654925238770426e-05</v>
       </c>
       <c r="G12">
-        <v>-2.4333501048798886e-05</v>
+        <v>2.6813406474502808e-07</v>
       </c>
       <c r="H12">
-        <v>-5.4849531344481478e-06</v>
+        <v>7.655752822538595e-06</v>
       </c>
       <c r="I12">
-        <v>8.2831097415042186e-05</v>
+        <v>2.3057124559346988e-05</v>
       </c>
       <c r="J12">
-        <v>-0.00045982538474761628</v>
+        <v>-6.5096680805900128e-05</v>
       </c>
       <c r="K12">
-        <v>1.0395485362990614e-05</v>
+        <v>-1.3639714086494223e-06</v>
       </c>
       <c r="L12">
-        <v>-4.0715320172183104e-06</v>
+        <v>2.2714633045317487e-06</v>
       </c>
       <c r="M12">
-        <v>0.00063883565286701439</v>
+        <v>7.5307071760238352e-05</v>
       </c>
       <c r="N12">
-        <v>9.4608499921825426e-06</v>
+        <v>-3.6634439352818961e-07</v>
       </c>
       <c r="O12">
-        <v>0.00045438385070667529</v>
+        <v>6.3710702773932295e-05</v>
       </c>
       <c r="P12">
-        <v>-0.00061142475532724656</v>
+        <v>-7.298279095239436e-05</v>
       </c>
       <c r="Q12">
-        <v>-0.00019866227728903326</v>
+        <v>-3.0928753385423572e-05</v>
       </c>
       <c r="R12">
-        <v>-0.00018411001790500124</v>
+        <v>-3.2786319386836512e-05</v>
       </c>
       <c r="S12">
-        <v>-0.0002257750330859217</v>
+        <v>-3.2591179853449747e-05</v>
       </c>
       <c r="T12">
-        <v>-3.6088427002290925e-05</v>
+        <v>-8.2752868392882915e-06</v>
       </c>
       <c r="U12">
-        <v>2.1954280476577358e-05</v>
+        <v>5.4532147123851329e-06</v>
       </c>
       <c r="V12">
-        <v>3.6938012733061165e-05</v>
+        <v>2.1209010254739871e-06</v>
       </c>
       <c r="W12">
-        <v>-2.3776958373916191e-05</v>
+        <v>-4.3790451813930481e-06</v>
       </c>
       <c r="X12">
-        <v>3.6866996768808093e-05</v>
+        <v>1.0492823791332157e-05</v>
       </c>
       <c r="Y12">
-        <v>-0.00019737655532720032</v>
+        <v>-3.5140046851827511e-05</v>
       </c>
       <c r="Z12">
-        <v>-5.2793343367700959e-05</v>
+        <v>-1.0553378979036472e-05</v>
       </c>
       <c r="AA12">
-        <v>-8.174737975831258e-05</v>
+        <v>-1.5697155095718355e-05</v>
       </c>
       <c r="AB12">
-        <v>-7.4798169395010197e-05</v>
+        <v>-1.7947351872157482e-05</v>
       </c>
       <c r="AC12">
-        <v>-6.6566042929599653e-05</v>
+        <v>-1.3303158559206591e-05</v>
       </c>
       <c r="AD12">
-        <v>-5.2188146467307259e-05</v>
+        <v>-1.1053181640752294e-05</v>
       </c>
       <c r="AE12">
-        <v>-5.4707719815161954e-05</v>
+        <v>-1.2242476380704357e-05</v>
       </c>
       <c r="AF12">
-        <v>4.5140438765156904e-06</v>
+        <v>1.1087454115216786e-06</v>
       </c>
       <c r="AG12">
-        <v>7.9398350037771e-05</v>
+        <v>1.290950570694912e-05</v>
       </c>
       <c r="AH12">
-        <v>5.0290009126370559e-05</v>
+        <v>1.3523503522019133e-05</v>
       </c>
       <c r="AI12">
-        <v>-0.00010912148249779828</v>
+        <v>-1.905461139721737e-05</v>
       </c>
     </row>
     <row r="13">
@@ -5622,106 +5622,106 @@
         <v>39</v>
       </c>
       <c r="B13">
-        <v>0.075677520889658234</v>
+        <v>0.045696865127133238</v>
       </c>
       <c r="C13">
-        <v>-0.00032709392055204717</v>
+        <v>-0.00024034260259612488</v>
       </c>
       <c r="D13">
-        <v>1.587768351397972e-06</v>
+        <v>3.1532069630658345e-07</v>
       </c>
       <c r="E13">
-        <v>-3.4959148584785588e-08</v>
+        <v>-1.7725946010885246e-08</v>
       </c>
       <c r="F13">
-        <v>-2.221052676966873e-05</v>
+        <v>-1.7393331160956826e-05</v>
       </c>
       <c r="G13">
-        <v>1.2426357628698525e-05</v>
+        <v>9.3865545268970109e-06</v>
       </c>
       <c r="H13">
-        <v>1.6768692062677903e-05</v>
+        <v>4.2859539845740394e-06</v>
       </c>
       <c r="I13">
-        <v>6.1195803712241507e-05</v>
+        <v>4.1849089375644254e-05</v>
       </c>
       <c r="J13">
-        <v>-2.3347955927411466e-05</v>
+        <v>-3.122888310336402e-06</v>
       </c>
       <c r="K13">
-        <v>1.7986021986654278e-05</v>
+        <v>1.3463637768981388e-05</v>
       </c>
       <c r="L13">
-        <v>8.4221969913879455e-07</v>
+        <v>5.0481052890735936e-07</v>
       </c>
       <c r="M13">
-        <v>9.4608499921825426e-06</v>
+        <v>-3.6634439352818961e-07</v>
       </c>
       <c r="N13">
-        <v>0.0074385457061766948</v>
+        <v>0.0054023609774367194</v>
       </c>
       <c r="O13">
-        <v>0.00012130999266770541</v>
+        <v>-0.00011392201719039749</v>
       </c>
       <c r="P13">
-        <v>0.0005783430327398031</v>
+        <v>0.00025355586642840188</v>
       </c>
       <c r="Q13">
-        <v>0.0044497253950711198</v>
+        <v>0.003143876566568251</v>
       </c>
       <c r="R13">
-        <v>0.0044441537076495424</v>
+        <v>0.0031367564315206318</v>
       </c>
       <c r="S13">
-        <v>0.0044151738506471444</v>
+        <v>0.0031138684658133182</v>
       </c>
       <c r="T13">
-        <v>0.00011822182869630467</v>
+        <v>0.00013469517750868939</v>
       </c>
       <c r="U13">
-        <v>3.3146942100654173e-05</v>
+        <v>2.0021917693776713e-05</v>
       </c>
       <c r="V13">
-        <v>0.00018222348271810547</v>
+        <v>0.00013139748255474302</v>
       </c>
       <c r="W13">
-        <v>-4.2543583907250739e-05</v>
+        <v>-3.3220939055277261e-05</v>
       </c>
       <c r="X13">
-        <v>-4.7090840577933713e-07</v>
+        <v>-9.1130213531504141e-06</v>
       </c>
       <c r="Y13">
-        <v>-0.00012331938187331941</v>
+        <v>-9.8619098376432311e-05</v>
       </c>
       <c r="Z13">
-        <v>6.3892697498914601e-05</v>
+        <v>0.00012401814429304544</v>
       </c>
       <c r="AA13">
-        <v>0.00011439383984365313</v>
+        <v>0.00016044528123872084</v>
       </c>
       <c r="AB13">
-        <v>0.00013461317724291501</v>
+        <v>0.00019725792838860698</v>
       </c>
       <c r="AC13">
-        <v>9.7898026577931821e-05</v>
+        <v>0.00014651550897268654</v>
       </c>
       <c r="AD13">
-        <v>7.1443082540535198e-05</v>
+        <v>0.00012474930381014453</v>
       </c>
       <c r="AE13">
-        <v>0.00012350157466021208</v>
+        <v>0.0001852813442095532</v>
       </c>
       <c r="AF13">
-        <v>-1.6835123396858036e-06</v>
+        <v>-5.421617844185672e-07</v>
       </c>
       <c r="AG13">
-        <v>6.7252230678467063e-05</v>
+        <v>3.2833001582458464e-05</v>
       </c>
       <c r="AH13">
-        <v>3.4368224754767647e-05</v>
+        <v>2.8941215185435436e-05</v>
       </c>
       <c r="AI13">
-        <v>-0.0044423224796542029</v>
+        <v>-0.003199411113164013</v>
       </c>
     </row>
     <row r="14">
@@ -5729,106 +5729,106 @@
         <v>66</v>
       </c>
       <c r="B14">
-        <v>-0.13662494003012624</v>
+        <v>-0.021116651853919446</v>
       </c>
       <c r="C14">
-        <v>-5.2614115386368898e-05</v>
+        <v>-1.0223419842135619e-05</v>
       </c>
       <c r="D14">
-        <v>4.7129042874799443e-06</v>
+        <v>-7.4091149670805026e-08</v>
       </c>
       <c r="E14">
-        <v>-3.8211111394579369e-08</v>
+        <v>2.2688116442150717e-09</v>
       </c>
       <c r="F14">
-        <v>-2.6264729022641535e-06</v>
+        <v>-1.0381919715457988e-05</v>
       </c>
       <c r="G14">
-        <v>2.7402438157772373e-05</v>
+        <v>5.0526528036755011e-06</v>
       </c>
       <c r="H14">
-        <v>5.8139325118979502e-05</v>
+        <v>2.0651020696011693e-05</v>
       </c>
       <c r="I14">
-        <v>0.00019333505088077983</v>
+        <v>3.8196819185115681e-05</v>
       </c>
       <c r="J14">
-        <v>-0.00063916565257824678</v>
+        <v>-7.5920632807978535e-05</v>
       </c>
       <c r="K14">
-        <v>2.3619129366459282e-05</v>
+        <v>2.7466930257796166e-06</v>
       </c>
       <c r="L14">
-        <v>-8.418638274399032e-06</v>
+        <v>1.094630901900406e-06</v>
       </c>
       <c r="M14">
-        <v>0.00045438385070667529</v>
+        <v>6.3710702773932295e-05</v>
       </c>
       <c r="N14">
-        <v>0.00012130999266770541</v>
+        <v>-0.00011392201719039749</v>
       </c>
       <c r="O14">
-        <v>0.01057464469854366</v>
+        <v>0.0012769543957204432</v>
       </c>
       <c r="P14">
-        <v>-0.0074848957076368372</v>
+        <v>-0.0010403094967339445</v>
       </c>
       <c r="Q14">
-        <v>0.0037722655307442371</v>
+        <v>0.00070658237498762351</v>
       </c>
       <c r="R14">
-        <v>0.0037716578152304607</v>
+        <v>0.00070660488532476575</v>
       </c>
       <c r="S14">
-        <v>0.0037326038703194338</v>
+        <v>0.00070660489949130642</v>
       </c>
       <c r="T14">
-        <v>6.799584020791556e-05</v>
+        <v>2.0022371290431254e-05</v>
       </c>
       <c r="U14">
-        <v>8.2907278544705921e-05</v>
+        <v>2.595289062499854e-05</v>
       </c>
       <c r="V14">
-        <v>0.00011489318579543873</v>
+        <v>2.6230948615721508e-05</v>
       </c>
       <c r="W14">
-        <v>-2.5224057276764082e-05</v>
+        <v>-3.8825774180729108e-06</v>
       </c>
       <c r="X14">
-        <v>6.0222017016385771e-05</v>
+        <v>1.7266261719943712e-05</v>
       </c>
       <c r="Y14">
-        <v>5.7313670718088842e-05</v>
+        <v>2.2703858386491338e-05</v>
       </c>
       <c r="Z14">
-        <v>-0.00011547568708166747</v>
+        <v>-4.1741491435329258e-05</v>
       </c>
       <c r="AA14">
-        <v>-9.553782629575147e-05</v>
+        <v>-3.7558632074420238e-05</v>
       </c>
       <c r="AB14">
-        <v>-0.00010038128288236559</v>
+        <v>-3.7989180969422463e-05</v>
       </c>
       <c r="AC14">
-        <v>-0.00012848653550902875</v>
+        <v>-4.6037538605574115e-05</v>
       </c>
       <c r="AD14">
-        <v>-4.7242070389820132e-05</v>
+        <v>-3.7540151969539556e-05</v>
       </c>
       <c r="AE14">
-        <v>-9.497152143127203e-05</v>
+        <v>-4.3420541572997698e-05</v>
       </c>
       <c r="AF14">
-        <v>-2.9833865790864454e-06</v>
+        <v>-7.1055333476091166e-07</v>
       </c>
       <c r="AG14">
-        <v>0.00017536319512749359</v>
+        <v>2.9504140180518852e-05</v>
       </c>
       <c r="AH14">
-        <v>0.00022196014127580637</v>
+        <v>3.4805187773936431e-05</v>
       </c>
       <c r="AI14">
-        <v>-0.0037023871339994029</v>
+        <v>-0.00066844723513465412</v>
       </c>
     </row>
     <row r="15">
@@ -5836,106 +5836,106 @@
         <v>67</v>
       </c>
       <c r="B15">
-        <v>0.042579154919832565</v>
+        <v>0.039770997714112993</v>
       </c>
       <c r="C15">
-        <v>3.3549356567971337e-05</v>
+        <v>4.576667820430703e-06</v>
       </c>
       <c r="D15">
-        <v>-2.2156869189074688e-06</v>
+        <v>2.7184789103790458e-07</v>
       </c>
       <c r="E15">
-        <v>2.4471266978375564e-08</v>
+        <v>-2.0261303533115006e-09</v>
       </c>
       <c r="F15">
-        <v>6.2568237371362192e-05</v>
+        <v>1.5451374548412723e-05</v>
       </c>
       <c r="G15">
-        <v>3.0600985372090765e-05</v>
+        <v>1.6942264189230539e-06</v>
       </c>
       <c r="H15">
-        <v>-6.8756435468558244e-06</v>
+        <v>-1.0737971898872799e-05</v>
       </c>
       <c r="I15">
-        <v>-0.00010390538640871693</v>
+        <v>-2.4508959900644691e-05</v>
       </c>
       <c r="J15">
-        <v>0.00043986487685248341</v>
+        <v>6.3305209309768443e-05</v>
       </c>
       <c r="K15">
-        <v>-9.4033853972996361e-06</v>
+        <v>1.2614631502436618e-06</v>
       </c>
       <c r="L15">
-        <v>4.6374156606388902e-06</v>
+        <v>-2.1465462890232318e-06</v>
       </c>
       <c r="M15">
-        <v>-0.00061142475532724656</v>
+        <v>-7.298279095239436e-05</v>
       </c>
       <c r="N15">
-        <v>0.0005783430327398031</v>
+        <v>0.00025355586642840188</v>
       </c>
       <c r="O15">
-        <v>-0.0074848957076368372</v>
+        <v>-0.0010403094967339445</v>
       </c>
       <c r="P15">
-        <v>0.009688435520830695</v>
+        <v>0.0012488559653919963</v>
       </c>
       <c r="Q15">
-        <v>0.0034900312782587726</v>
+        <v>0.0010167608927740242</v>
       </c>
       <c r="R15">
-        <v>0.0034798574403264483</v>
+        <v>0.001019554288409</v>
       </c>
       <c r="S15">
-        <v>0.0035207377562913172</v>
+        <v>0.001018056860376293</v>
       </c>
       <c r="T15">
-        <v>-2.8474912227118834e-05</v>
+        <v>-1.8396627539396591e-05</v>
       </c>
       <c r="U15">
-        <v>-1.0017500246774203e-05</v>
+        <v>-5.3823427814128568e-06</v>
       </c>
       <c r="V15">
-        <v>-2.4610251780634695e-05</v>
+        <v>-1.8199951561626254e-06</v>
       </c>
       <c r="W15">
-        <v>2.3697218473121755e-05</v>
+        <v>3.9921339113148423e-06</v>
       </c>
       <c r="X15">
-        <v>-3.7255878129687707e-05</v>
+        <v>-1.0195612902429526e-05</v>
       </c>
       <c r="Y15">
-        <v>0.00016661892369636234</v>
+        <v>2.316996492159111e-05</v>
       </c>
       <c r="Z15">
-        <v>8.6525314375642546e-05</v>
+        <v>2.8500856413521142e-05</v>
       </c>
       <c r="AA15">
-        <v>0.00010835578757822277</v>
+        <v>3.1628420065588504e-05</v>
       </c>
       <c r="AB15">
-        <v>8.8851153156342948e-05</v>
+        <v>3.4950511344949709e-05</v>
       </c>
       <c r="AC15">
-        <v>0.00010941218739209991</v>
+        <v>3.1764693548203232e-05</v>
       </c>
       <c r="AD15">
-        <v>6.8524030885496129e-05</v>
+        <v>2.9113856266219703e-05</v>
       </c>
       <c r="AE15">
-        <v>5.8228554816225743e-05</v>
+        <v>2.6371509084704827e-05</v>
       </c>
       <c r="AF15">
-        <v>-4.835728867982459e-06</v>
+        <v>-1.0920358114035344e-06</v>
       </c>
       <c r="AG15">
-        <v>-4.5397950292241571e-05</v>
+        <v>-5.9418637690063832e-06</v>
       </c>
       <c r="AH15">
-        <v>-0.00015119055836303815</v>
+        <v>-2.8616771146732921e-05</v>
       </c>
       <c r="AI15">
-        <v>-0.0031849625751416287</v>
+        <v>-0.00097849154912832176</v>
       </c>
     </row>
     <row r="16">
@@ -5943,106 +5943,106 @@
         <v>43</v>
       </c>
       <c r="B16">
-        <v>-0.27858390856768867</v>
+        <v>-0.041524420204073466</v>
       </c>
       <c r="C16">
-        <v>-0.00023316230487734562</v>
+        <v>-0.00018675253873414515</v>
       </c>
       <c r="D16">
-        <v>-2.4718436714475417e-05</v>
+        <v>-2.0730517857023458e-05</v>
       </c>
       <c r="E16">
-        <v>1.5717468542467302e-07</v>
+        <v>1.345105398685577e-07</v>
       </c>
       <c r="F16">
-        <v>3.4086789976513036e-05</v>
+        <v>-1.6462071217785649e-05</v>
       </c>
       <c r="G16">
-        <v>0.00011215392557799037</v>
+        <v>5.0933515410422209e-05</v>
       </c>
       <c r="H16">
-        <v>0.00012172266110459327</v>
+        <v>6.7345411768237901e-05</v>
       </c>
       <c r="I16">
-        <v>0.0002252244350126123</v>
+        <v>0.00013209345152957091</v>
       </c>
       <c r="J16">
-        <v>-0.00028121560836039735</v>
+        <v>-4.53730621217587e-05</v>
       </c>
       <c r="K16">
-        <v>0.00011245365347632881</v>
+        <v>8.8838302483919577e-05</v>
       </c>
       <c r="L16">
-        <v>-8.4233950044148215e-06</v>
+        <v>-5.2446072122630411e-06</v>
       </c>
       <c r="M16">
-        <v>-0.00019866227728903326</v>
+        <v>-3.0928753385423572e-05</v>
       </c>
       <c r="N16">
-        <v>0.0044497253950711198</v>
+        <v>0.003143876566568251</v>
       </c>
       <c r="O16">
-        <v>0.0037722655307442371</v>
+        <v>0.00070658237498762351</v>
       </c>
       <c r="P16">
-        <v>0.0034900312782587726</v>
+        <v>0.0010167608927740242</v>
       </c>
       <c r="Q16">
-        <v>0.016755690848965166</v>
+        <v>0.012008777553138766</v>
       </c>
       <c r="R16">
-        <v>0.016320488162909159</v>
+        <v>0.011695797723531931</v>
       </c>
       <c r="S16">
-        <v>0.016299966950468654</v>
+        <v>0.011669206246228572</v>
       </c>
       <c r="T16">
-        <v>0.003600202638976196</v>
+        <v>0.0029771787142031441</v>
       </c>
       <c r="U16">
-        <v>0.00067584595036841548</v>
+        <v>0.00054304833169308182</v>
       </c>
       <c r="V16">
-        <v>0.00084114758004532491</v>
+        <v>0.0006671776916946379</v>
       </c>
       <c r="W16">
-        <v>-4.4052120864641406e-05</v>
+        <v>-3.5816147462752225e-05</v>
       </c>
       <c r="X16">
-        <v>2.9757273650001578e-05</v>
+        <v>1.7291944555928923e-05</v>
       </c>
       <c r="Y16">
-        <v>0.00023147393001431062</v>
+        <v>0.0001220726888068787</v>
       </c>
       <c r="Z16">
-        <v>-1.4248406050923479e-05</v>
+        <v>6.6182500210149042e-05</v>
       </c>
       <c r="AA16">
-        <v>4.6359194890806775e-05</v>
+        <v>9.487294352295006e-05</v>
       </c>
       <c r="AB16">
-        <v>9.9282122083284253e-05</v>
+        <v>0.00015783475030169613</v>
       </c>
       <c r="AC16">
-        <v>-3.4653852526901445e-05</v>
+        <v>3.0762400758397104e-05</v>
       </c>
       <c r="AD16">
-        <v>6.5856619127423362e-05</v>
+        <v>0.00011287110516250659</v>
       </c>
       <c r="AE16">
-        <v>-4.8637700066664173e-07</v>
+        <v>7.3446356314997813e-05</v>
       </c>
       <c r="AF16">
-        <v>-4.2407887498384193e-06</v>
+        <v>-4.8402692097325375e-07</v>
       </c>
       <c r="AG16">
-        <v>0.00031659723868952827</v>
+        <v>0.00019026094556276463</v>
       </c>
       <c r="AH16">
-        <v>0.00019594872205736056</v>
+        <v>9.7376897196153021e-05</v>
       </c>
       <c r="AI16">
-        <v>-0.015825749025517082</v>
+        <v>-0.011551297423127107</v>
       </c>
     </row>
     <row r="17">
@@ -6050,106 +6050,106 @@
         <v>44</v>
       </c>
       <c r="B17">
-        <v>-0.21378754484854434</v>
+        <v>-0.0089967538258947082</v>
       </c>
       <c r="C17">
-        <v>-0.00023008438428831932</v>
+        <v>-0.00018151597747181135</v>
       </c>
       <c r="D17">
-        <v>-3.6741172482691127e-05</v>
+        <v>-2.9683770745107406e-05</v>
       </c>
       <c r="E17">
-        <v>2.9121799219837417e-07</v>
+        <v>2.3201903387752886e-07</v>
       </c>
       <c r="F17">
-        <v>9.2686772673516125e-05</v>
+        <v>2.7511439242178248e-05</v>
       </c>
       <c r="G17">
-        <v>0.00010674103557494451</v>
+        <v>4.1964274798717439e-05</v>
       </c>
       <c r="H17">
-        <v>9.4734495009401488e-05</v>
+        <v>4.35244828016065e-05</v>
       </c>
       <c r="I17">
-        <v>0.00022811049602714829</v>
+        <v>0.00012728769464689796</v>
       </c>
       <c r="J17">
-        <v>-0.00028120091219737076</v>
+        <v>-4.4683056230358801e-05</v>
       </c>
       <c r="K17">
-        <v>8.4701074168258951e-05</v>
+        <v>6.2896581643416809e-05</v>
       </c>
       <c r="L17">
-        <v>-2.4807567488618741e-05</v>
+        <v>-1.8481287009426216e-05</v>
       </c>
       <c r="M17">
-        <v>-0.00018411001790500124</v>
+        <v>-3.2786319386836512e-05</v>
       </c>
       <c r="N17">
-        <v>0.0044441537076495424</v>
+        <v>0.0031367564315206318</v>
       </c>
       <c r="O17">
-        <v>0.0037716578152304607</v>
+        <v>0.00070660488532476575</v>
       </c>
       <c r="P17">
-        <v>0.0034798574403264483</v>
+        <v>0.001019554288409</v>
       </c>
       <c r="Q17">
-        <v>0.016320488162909159</v>
+        <v>0.011695797723531931</v>
       </c>
       <c r="R17">
-        <v>0.016582958235566887</v>
+        <v>0.011894305970167749</v>
       </c>
       <c r="S17">
-        <v>0.016165211278795173</v>
+        <v>0.011579020506819346</v>
       </c>
       <c r="T17">
-        <v>0.0030999572069719526</v>
+        <v>0.0025435265004966432</v>
       </c>
       <c r="U17">
-        <v>0.00040240943404083913</v>
+        <v>0.00028300368417480751</v>
       </c>
       <c r="V17">
-        <v>0.0005256087312728345</v>
+        <v>0.00038790812345809115</v>
       </c>
       <c r="W17">
-        <v>-6.0744806840123128e-05</v>
+        <v>-5.1554931737010667e-05</v>
       </c>
       <c r="X17">
-        <v>-5.1193897151529874e-06</v>
+        <v>-1.7823892669612852e-05</v>
       </c>
       <c r="Y17">
-        <v>9.3570909470648382e-05</v>
+        <v>5.2840393465285705e-06</v>
       </c>
       <c r="Z17">
-        <v>9.9286993257364023e-06</v>
+        <v>6.7856582924429899e-05</v>
       </c>
       <c r="AA17">
-        <v>6.572844696292211e-05</v>
+        <v>0.00010159802617199822</v>
       </c>
       <c r="AB17">
-        <v>7.9839508586744285e-05</v>
+        <v>0.00013175722019482779</v>
       </c>
       <c r="AC17">
-        <v>1.0444425434076934e-05</v>
+        <v>5.4821079419653182e-05</v>
       </c>
       <c r="AD17">
-        <v>8.7148450729574757e-05</v>
+        <v>0.00011607455231191243</v>
       </c>
       <c r="AE17">
-        <v>3.6249155061806844e-05</v>
+        <v>9.5597050472739378e-05</v>
       </c>
       <c r="AF17">
-        <v>-8.6701134686602592e-06</v>
+        <v>-3.8478896559055505e-06</v>
       </c>
       <c r="AG17">
-        <v>0.0002879989900816636</v>
+        <v>0.00016438269767595284</v>
       </c>
       <c r="AH17">
-        <v>0.0001867011565983975</v>
+        <v>9.4695687023475111e-05</v>
       </c>
       <c r="AI17">
-        <v>-0.01502158810750011</v>
+        <v>-0.0108666916165113</v>
       </c>
     </row>
     <row r="18">
@@ -6157,106 +6157,106 @@
         <v>45</v>
       </c>
       <c r="B18">
-        <v>-0.1249114686515805</v>
+        <v>0.047190442355942955</v>
       </c>
       <c r="C18">
-        <v>-0.00019367918701796553</v>
+        <v>-0.00015507529010086275</v>
       </c>
       <c r="D18">
-        <v>-2.7618385373603016e-05</v>
+        <v>-2.1545048505077787e-05</v>
       </c>
       <c r="E18">
-        <v>2.2981023190497959e-07</v>
+        <v>1.7713008708386214e-07</v>
       </c>
       <c r="F18">
-        <v>7.234623004049234e-05</v>
+        <v>1.4456196281646683e-05</v>
       </c>
       <c r="G18">
-        <v>0.00010523337934325834</v>
+        <v>4.6691616419018874e-05</v>
       </c>
       <c r="H18">
-        <v>7.388652170449081e-05</v>
+        <v>3.690571616251628e-05</v>
       </c>
       <c r="I18">
-        <v>0.00013170444398262395</v>
+        <v>6.5374092568053471e-05</v>
       </c>
       <c r="J18">
-        <v>-0.00024159070326182217</v>
+        <v>-4.337675529428107e-05</v>
       </c>
       <c r="K18">
-        <v>1.2075251853831039e-05</v>
+        <v>9.5007338137436705e-06</v>
       </c>
       <c r="L18">
-        <v>-1.1985930145395562e-05</v>
+        <v>-6.0486556435260163e-06</v>
       </c>
       <c r="M18">
-        <v>-0.0002257750330859217</v>
+        <v>-3.2591179853449747e-05</v>
       </c>
       <c r="N18">
-        <v>0.0044151738506471444</v>
+        <v>0.0031138684658133182</v>
       </c>
       <c r="O18">
-        <v>0.0037326038703194338</v>
+        <v>0.00070660489949130642</v>
       </c>
       <c r="P18">
-        <v>0.0035207377562913172</v>
+        <v>0.001018056860376293</v>
       </c>
       <c r="Q18">
-        <v>0.016299966950468654</v>
+        <v>0.011669206246228572</v>
       </c>
       <c r="R18">
-        <v>0.016165211278795173</v>
+        <v>0.011579020506819346</v>
       </c>
       <c r="S18">
-        <v>0.016408465661292653</v>
+        <v>0.011747020299627424</v>
       </c>
       <c r="T18">
-        <v>0.0028197971898799128</v>
+        <v>0.002365847834919511</v>
       </c>
       <c r="U18">
-        <v>-2.5275215848472726e-05</v>
+        <v>-9.3612752841117433e-06</v>
       </c>
       <c r="V18">
-        <v>3.2504609520023686e-05</v>
+        <v>4.1114775312971023e-05</v>
       </c>
       <c r="W18">
-        <v>-6.731041884144413e-05</v>
+        <v>-5.4361942385244334e-05</v>
       </c>
       <c r="X18">
-        <v>-2.1592972747274189e-05</v>
+        <v>-1.6540941160553139e-05</v>
       </c>
       <c r="Y18">
-        <v>0.00021078688298528658</v>
+        <v>0.0001029112026425011</v>
       </c>
       <c r="Z18">
-        <v>-1.6892185388245676e-05</v>
+        <v>1.5977289439899484e-05</v>
       </c>
       <c r="AA18">
-        <v>4.3026856138298538e-05</v>
+        <v>4.9367833054357949e-05</v>
       </c>
       <c r="AB18">
-        <v>7.0954999775664626e-05</v>
+        <v>8.5799646120243581e-05</v>
       </c>
       <c r="AC18">
-        <v>-6.8574665755454303e-06</v>
+        <v>6.352830463492512e-06</v>
       </c>
       <c r="AD18">
-        <v>5.9035760047622746e-05</v>
+        <v>5.9201836919625228e-05</v>
       </c>
       <c r="AE18">
-        <v>1.7587982876780405e-05</v>
+        <v>4.3467628110373442e-05</v>
       </c>
       <c r="AF18">
-        <v>-1.1447210369927276e-05</v>
+        <v>-6.1333967309722153e-06</v>
       </c>
       <c r="AG18">
-        <v>0.0002006316169769623</v>
+        <v>0.0001026237763215327</v>
       </c>
       <c r="AH18">
-        <v>0.00014512875049894208</v>
+        <v>7.1503295263667353e-05</v>
       </c>
       <c r="AI18">
-        <v>-0.014763368816508946</v>
+        <v>-0.010715118799295528</v>
       </c>
     </row>
     <row r="19">
@@ -6264,106 +6264,106 @@
         <v>46</v>
       </c>
       <c r="B19">
-        <v>0.30689102994222972</v>
+        <v>0.22675041138778157</v>
       </c>
       <c r="C19">
-        <v>-0.0001027422881938953</v>
+        <v>-9.5660569266283366e-05</v>
       </c>
       <c r="D19">
-        <v>5.6327917884880805e-05</v>
+        <v>4.1911041234563763e-05</v>
       </c>
       <c r="E19">
-        <v>-5.3255137979159031e-07</v>
+        <v>-3.9850582766799807e-07</v>
       </c>
       <c r="F19">
-        <v>0.00010735315558156209</v>
+        <v>7.2319497612602108e-05</v>
       </c>
       <c r="G19">
-        <v>6.506798789906185e-05</v>
+        <v>6.1135750738960503e-05</v>
       </c>
       <c r="H19">
-        <v>6.3292858309631217e-05</v>
+        <v>1.7097488510219461e-05</v>
       </c>
       <c r="I19">
-        <v>-0.00013543921931975181</v>
+        <v>-8.2717081325280224e-05</v>
       </c>
       <c r="J19">
-        <v>-5.9662954073992389e-05</v>
+        <v>-1.2158462172536947e-05</v>
       </c>
       <c r="K19">
-        <v>0.0024972211811194393</v>
+        <v>0.0018872080951591495</v>
       </c>
       <c r="L19">
-        <v>-4.933522852928612e-05</v>
+        <v>-4.1690923457297036e-05</v>
       </c>
       <c r="M19">
-        <v>-3.6088427002290925e-05</v>
+        <v>-8.2752868392882915e-06</v>
       </c>
       <c r="N19">
-        <v>0.00011822182869630467</v>
+        <v>0.00013469517750868939</v>
       </c>
       <c r="O19">
-        <v>6.799584020791556e-05</v>
+        <v>2.0022371290431254e-05</v>
       </c>
       <c r="P19">
-        <v>-2.8474912227118834e-05</v>
+        <v>-1.8396627539396591e-05</v>
       </c>
       <c r="Q19">
-        <v>0.003600202638976196</v>
+        <v>0.0029771787142031441</v>
       </c>
       <c r="R19">
-        <v>0.0030999572069719526</v>
+        <v>0.0025435265004966432</v>
       </c>
       <c r="S19">
-        <v>0.0028197971898799128</v>
+        <v>0.002365847834919511</v>
       </c>
       <c r="T19">
-        <v>0.023718959018883545</v>
+        <v>0.018073448140702914</v>
       </c>
       <c r="U19">
-        <v>0.020014447954107284</v>
+        <v>0.01511653657210689</v>
       </c>
       <c r="V19">
-        <v>0.020148993634667056</v>
+        <v>0.015229920627762718</v>
       </c>
       <c r="W19">
-        <v>3.4522939287826981e-05</v>
+        <v>7.0611643962856284e-05</v>
       </c>
       <c r="X19">
-        <v>2.190562178820514e-05</v>
+        <v>9.8248452292374992e-05</v>
       </c>
       <c r="Y19">
-        <v>0.0007232136229608525</v>
+        <v>0.00070207492734455923</v>
       </c>
       <c r="Z19">
-        <v>-2.1245397239001707e-06</v>
+        <v>8.1796134884655827e-05</v>
       </c>
       <c r="AA19">
-        <v>-0.00023697175779435059</v>
+        <v>-6.5977748268545265e-05</v>
       </c>
       <c r="AB19">
-        <v>-0.00023627816261422669</v>
+        <v>-8.1554675259494763e-05</v>
       </c>
       <c r="AC19">
-        <v>-4.9982022240475585e-05</v>
+        <v>5.5011388798308428e-05</v>
       </c>
       <c r="AD19">
-        <v>-0.00029799213440012858</v>
+        <v>-0.00010304340954919852</v>
       </c>
       <c r="AE19">
-        <v>-6.9971695066448243e-05</v>
+        <v>-8.9685666702423459e-05</v>
       </c>
       <c r="AF19">
-        <v>2.1528153876205439e-07</v>
+        <v>2.9647257412071418e-06</v>
       </c>
       <c r="AG19">
-        <v>-5.5994886211566119e-05</v>
+        <v>-6.2888099250091312e-06</v>
       </c>
       <c r="AH19">
-        <v>0.00014858609909701621</v>
+        <v>1.4120930301418644e-05</v>
       </c>
       <c r="AI19">
-        <v>-0.024416804220154135</v>
+        <v>-0.018831810835430202</v>
       </c>
     </row>
     <row r="20">
@@ -6371,106 +6371,106 @@
         <v>47</v>
       </c>
       <c r="B20">
-        <v>0.26153167700082769</v>
+        <v>0.24438362484980597</v>
       </c>
       <c r="C20">
-        <v>-5.2265305761841304e-05</v>
+        <v>-2.95200541884232e-05</v>
       </c>
       <c r="D20">
-        <v>-2.8715351058527014e-05</v>
+        <v>-2.4552717071218503e-05</v>
       </c>
       <c r="E20">
-        <v>9.3323005600879071e-08</v>
+        <v>8.5366265271832758e-08</v>
       </c>
       <c r="F20">
-        <v>0.00013435923948253528</v>
+        <v>8.6116183005344616e-05</v>
       </c>
       <c r="G20">
-        <v>0.00011380341857671148</v>
+        <v>9.7678731807014207e-05</v>
       </c>
       <c r="H20">
-        <v>0.00014956025952320585</v>
+        <v>9.7737619638381271e-05</v>
       </c>
       <c r="I20">
-        <v>-6.0851686910935905e-05</v>
+        <v>-5.4794783141643485e-05</v>
       </c>
       <c r="J20">
-        <v>-9.3223257890432193e-05</v>
+        <v>-2.7260263517076077e-05</v>
       </c>
       <c r="K20">
-        <v>0.0025423143104802422</v>
+        <v>0.0019220082482929528</v>
       </c>
       <c r="L20">
-        <v>-6.637102713381732e-05</v>
+        <v>-4.9678699126256522e-05</v>
       </c>
       <c r="M20">
-        <v>2.1954280476577358e-05</v>
+        <v>5.4532147123851329e-06</v>
       </c>
       <c r="N20">
-        <v>3.3146942100654173e-05</v>
+        <v>2.0021917693776713e-05</v>
       </c>
       <c r="O20">
-        <v>8.2907278544705921e-05</v>
+        <v>2.595289062499854e-05</v>
       </c>
       <c r="P20">
-        <v>-1.0017500246774203e-05</v>
+        <v>-5.3823427814128568e-06</v>
       </c>
       <c r="Q20">
-        <v>0.00067584595036841548</v>
+        <v>0.00054304833169308182</v>
       </c>
       <c r="R20">
-        <v>0.00040240943404083913</v>
+        <v>0.00028300368417480751</v>
       </c>
       <c r="S20">
-        <v>-2.5275215848472726e-05</v>
+        <v>-9.3612752841117433e-06</v>
       </c>
       <c r="T20">
-        <v>0.020014447954107284</v>
+        <v>0.01511653657210689</v>
       </c>
       <c r="U20">
-        <v>0.020715823942641615</v>
+        <v>0.015723565725514799</v>
       </c>
       <c r="V20">
-        <v>0.020655427483198725</v>
+        <v>0.015679695076591789</v>
       </c>
       <c r="W20">
-        <v>-0.00012790703301523485</v>
+        <v>-6.8321306906789572e-05</v>
       </c>
       <c r="X20">
-        <v>2.8191657824618455e-05</v>
+        <v>9.1066052044852259e-05</v>
       </c>
       <c r="Y20">
-        <v>0.00051999392204682676</v>
+        <v>0.00057607957093675508</v>
       </c>
       <c r="Z20">
-        <v>6.6557231107324325e-05</v>
+        <v>0.00018260500360920383</v>
       </c>
       <c r="AA20">
-        <v>-0.00015827837842209442</v>
+        <v>4.8086735575649138e-05</v>
       </c>
       <c r="AB20">
-        <v>-0.00021599875091771149</v>
+        <v>-5.1239361966075401e-06</v>
       </c>
       <c r="AC20">
-        <v>5.6598753435136047e-05</v>
+        <v>0.00019026714922081717</v>
       </c>
       <c r="AD20">
-        <v>-0.00021078048529140064</v>
+        <v>3.853106959384768e-07</v>
       </c>
       <c r="AE20">
-        <v>6.7585007183653626e-05</v>
+        <v>9.3167404871446384e-05</v>
       </c>
       <c r="AF20">
-        <v>6.9688415398830176e-06</v>
+        <v>7.4139764138646432e-06</v>
       </c>
       <c r="AG20">
-        <v>2.6878304278842719e-05</v>
+        <v>7.9994971644315252e-05</v>
       </c>
       <c r="AH20">
-        <v>0.00015217774312469186</v>
+        <v>1.3543670851434708e-05</v>
       </c>
       <c r="AI20">
-        <v>-0.019556821768951863</v>
+        <v>-0.014929297964842797</v>
       </c>
     </row>
     <row r="21">
@@ -6478,106 +6478,106 @@
         <v>48</v>
       </c>
       <c r="B21">
-        <v>0.31668596663367216</v>
+        <v>0.2819906190925453</v>
       </c>
       <c r="C21">
-        <v>-0.00020319985945792786</v>
+        <v>-0.00014176747662271859</v>
       </c>
       <c r="D21">
-        <v>-3.3873129909836963e-06</v>
+        <v>-8.3669400091756764e-06</v>
       </c>
       <c r="E21">
-        <v>-3.0831760440807579e-07</v>
+        <v>-1.8236208065779914e-07</v>
       </c>
       <c r="F21">
-        <v>3.649228354062322e-05</v>
+        <v>3.9381120078241195e-05</v>
       </c>
       <c r="G21">
-        <v>6.7121795603022763e-05</v>
+        <v>8.3261361007281199e-05</v>
       </c>
       <c r="H21">
-        <v>6.0869248048411742e-05</v>
+        <v>3.8233718438623193e-05</v>
       </c>
       <c r="I21">
-        <v>-0.00012846647571950452</v>
+        <v>-9.1353798657312774e-05</v>
       </c>
       <c r="J21">
-        <v>-0.00012104402601295762</v>
+        <v>-2.7004610335824979e-05</v>
       </c>
       <c r="K21">
-        <v>0.002568404299279205</v>
+        <v>0.0019437705410297766</v>
       </c>
       <c r="L21">
-        <v>-5.8997845047084071e-05</v>
+        <v>-4.723236331971339e-05</v>
       </c>
       <c r="M21">
-        <v>3.6938012733061165e-05</v>
+        <v>2.1209010254739871e-06</v>
       </c>
       <c r="N21">
-        <v>0.00018222348271810547</v>
+        <v>0.00013139748255474302</v>
       </c>
       <c r="O21">
-        <v>0.00011489318579543873</v>
+        <v>2.6230948615721508e-05</v>
       </c>
       <c r="P21">
-        <v>-2.4610251780634695e-05</v>
+        <v>-1.8199951561626254e-06</v>
       </c>
       <c r="Q21">
-        <v>0.00084114758004532491</v>
+        <v>0.0006671776916946379</v>
       </c>
       <c r="R21">
-        <v>0.0005256087312728345</v>
+        <v>0.00038790812345809115</v>
       </c>
       <c r="S21">
-        <v>3.2504609520023686e-05</v>
+        <v>4.1114775312971023e-05</v>
       </c>
       <c r="T21">
-        <v>0.020148993634667056</v>
+        <v>0.015229920627762718</v>
       </c>
       <c r="U21">
-        <v>0.020655427483198725</v>
+        <v>0.015679695076591789</v>
       </c>
       <c r="V21">
-        <v>0.021712917151899276</v>
+        <v>0.016426119721242243</v>
       </c>
       <c r="W21">
-        <v>-0.00015955138939490609</v>
+        <v>-0.00010476350483751729</v>
       </c>
       <c r="X21">
-        <v>2.2910447972973938e-05</v>
+        <v>5.8590977754004788e-05</v>
       </c>
       <c r="Y21">
-        <v>0.00049063200750470645</v>
+        <v>0.00053790788706125064</v>
       </c>
       <c r="Z21">
-        <v>3.2379196705672499e-05</v>
+        <v>0.00020058416387127957</v>
       </c>
       <c r="AA21">
-        <v>-0.00019517041910760771</v>
+        <v>7.8774566333253936e-05</v>
       </c>
       <c r="AB21">
-        <v>-0.0002307304293205051</v>
+        <v>3.6505203233518167e-05</v>
       </c>
       <c r="AC21">
-        <v>5.0429980654251652e-05</v>
+        <v>0.00023111009227154682</v>
       </c>
       <c r="AD21">
-        <v>-0.00023556963315815062</v>
+        <v>2.4134375351770807e-05</v>
       </c>
       <c r="AE21">
-        <v>5.9506652066179883e-05</v>
+        <v>0.0001348805627858201</v>
       </c>
       <c r="AF21">
-        <v>7.0868702618841553e-06</v>
+        <v>7.1148461006115976e-06</v>
       </c>
       <c r="AG21">
-        <v>9.5301536831786382e-05</v>
+        <v>0.00010872160819264814</v>
       </c>
       <c r="AH21">
-        <v>0.00019727308075736388</v>
+        <v>7.3259343357217656e-05</v>
       </c>
       <c r="AI21">
-        <v>-0.019970339422381342</v>
+        <v>-0.015225895337582101</v>
       </c>
     </row>
     <row r="22">
@@ -6585,106 +6585,106 @@
         <v>49</v>
       </c>
       <c r="B22">
-        <v>0.0094792007980459142</v>
+        <v>-0.0055814200925311695</v>
       </c>
       <c r="C22">
-        <v>4.0345429562238022e-05</v>
+        <v>2.9154778942572579e-05</v>
       </c>
       <c r="D22">
-        <v>8.9916027705526815e-06</v>
+        <v>1.0149484608886576e-05</v>
       </c>
       <c r="E22">
-        <v>-2.5385119997845615e-08</v>
+        <v>-4.687240301874925e-08</v>
       </c>
       <c r="F22">
-        <v>1.396123948230936e-06</v>
+        <v>-2.3705830900374821e-05</v>
       </c>
       <c r="G22">
-        <v>3.240480365034445e-05</v>
+        <v>9.8725724469550351e-06</v>
       </c>
       <c r="H22">
-        <v>1.4386862176733667e-05</v>
+        <v>-8.5563527611985386e-06</v>
       </c>
       <c r="I22">
-        <v>2.8852205235416919e-06</v>
+        <v>-1.1666824654228198e-05</v>
       </c>
       <c r="J22">
-        <v>2.2253769112660799e-05</v>
+        <v>2.7620788434536656e-06</v>
       </c>
       <c r="K22">
-        <v>-2.8229001594775981e-05</v>
+        <v>-1.9221651197954986e-05</v>
       </c>
       <c r="L22">
-        <v>2.1549592304919692e-07</v>
+        <v>9.2883273672897568e-09</v>
       </c>
       <c r="M22">
-        <v>-2.3776958373916191e-05</v>
+        <v>-4.3790451813930481e-06</v>
       </c>
       <c r="N22">
-        <v>-4.2543583907250739e-05</v>
+        <v>-3.3220939055277261e-05</v>
       </c>
       <c r="O22">
-        <v>-2.5224057276764082e-05</v>
+        <v>-3.8825774180729108e-06</v>
       </c>
       <c r="P22">
-        <v>2.3697218473121755e-05</v>
+        <v>3.9921339113148423e-06</v>
       </c>
       <c r="Q22">
-        <v>-4.4052120864641406e-05</v>
+        <v>-3.5816147462752225e-05</v>
       </c>
       <c r="R22">
-        <v>-6.0744806840123128e-05</v>
+        <v>-5.1554931737010667e-05</v>
       </c>
       <c r="S22">
-        <v>-6.731041884144413e-05</v>
+        <v>-5.4361942385244334e-05</v>
       </c>
       <c r="T22">
-        <v>3.4522939287826981e-05</v>
+        <v>7.0611643962856284e-05</v>
       </c>
       <c r="U22">
-        <v>-0.00012790703301523485</v>
+        <v>-6.8321306906789572e-05</v>
       </c>
       <c r="V22">
-        <v>-0.00015955138939490609</v>
+        <v>-0.00010476350483751729</v>
       </c>
       <c r="W22">
-        <v>0.00063219260239416608</v>
+        <v>0.00047555179875446426</v>
       </c>
       <c r="X22">
-        <v>0.00021111983175499925</v>
+        <v>0.00016636127862838999</v>
       </c>
       <c r="Y22">
-        <v>0.00032374727392850693</v>
+        <v>0.00025073862351095399</v>
       </c>
       <c r="Z22">
-        <v>-2.8259794567796529e-07</v>
+        <v>1.1209677716053802e-05</v>
       </c>
       <c r="AA22">
-        <v>-1.2850461832927804e-05</v>
+        <v>3.0164766362266756e-06</v>
       </c>
       <c r="AB22">
-        <v>8.9035697779476348e-07</v>
+        <v>1.6215172945386385e-05</v>
       </c>
       <c r="AC22">
-        <v>-6.1956261635208589e-06</v>
+        <v>8.347343052448163e-06</v>
       </c>
       <c r="AD22">
-        <v>7.9580214339586058e-06</v>
+        <v>1.8218598874120664e-05</v>
       </c>
       <c r="AE22">
-        <v>-5.1787848250889523e-05</v>
+        <v>-4.794041635996373e-05</v>
       </c>
       <c r="AF22">
-        <v>-1.6556312024076805e-08</v>
+        <v>-3.8638261772101368e-07</v>
       </c>
       <c r="AG22">
-        <v>3.3973305414521386e-05</v>
+        <v>3.4010345848732202e-05</v>
       </c>
       <c r="AH22">
-        <v>-1.182606046036495e-05</v>
+        <v>-1.6129807065460138e-05</v>
       </c>
       <c r="AI22">
-        <v>-0.00042718926414069328</v>
+        <v>-0.00041631372711569385</v>
       </c>
     </row>
     <row r="23">
@@ -6692,106 +6692,106 @@
         <v>50</v>
       </c>
       <c r="B23">
-        <v>0.076294703820031354</v>
+        <v>0.042900599829082231</v>
       </c>
       <c r="C23">
-        <v>-3.6891271348568258e-07</v>
+        <v>6.1134543296815869e-06</v>
       </c>
       <c r="D23">
-        <v>3.4925405800941836e-05</v>
+        <v>2.6659730312490085e-05</v>
       </c>
       <c r="E23">
-        <v>-2.8087293733730018e-07</v>
+        <v>-2.0757740691395408e-07</v>
       </c>
       <c r="F23">
-        <v>-1.148587195645874e-05</v>
+        <v>-3.3536093379019387e-05</v>
       </c>
       <c r="G23">
-        <v>3.6184796380715366e-05</v>
+        <v>1.1602479155745776e-05</v>
       </c>
       <c r="H23">
-        <v>2.9644530535361414e-05</v>
+        <v>6.5853044540289691e-06</v>
       </c>
       <c r="I23">
-        <v>7.5507397100281742e-05</v>
+        <v>4.6188312691185078e-05</v>
       </c>
       <c r="J23">
-        <v>-5.9665466520087527e-05</v>
+        <v>-1.8224339906499334e-05</v>
       </c>
       <c r="K23">
-        <v>2.2909570554582198e-06</v>
+        <v>7.4496682716483891e-06</v>
       </c>
       <c r="L23">
-        <v>2.8208978696641841e-06</v>
+        <v>3.5352631715359018e-06</v>
       </c>
       <c r="M23">
-        <v>3.6866996768808093e-05</v>
+        <v>1.0492823791332157e-05</v>
       </c>
       <c r="N23">
-        <v>-4.7090840577933713e-07</v>
+        <v>-9.1130213531504141e-06</v>
       </c>
       <c r="O23">
-        <v>6.0222017016385771e-05</v>
+        <v>1.7266261719943712e-05</v>
       </c>
       <c r="P23">
-        <v>-3.7255878129687707e-05</v>
+        <v>-1.0195612902429526e-05</v>
       </c>
       <c r="Q23">
-        <v>2.9757273650001578e-05</v>
+        <v>1.7291944555928923e-05</v>
       </c>
       <c r="R23">
-        <v>-5.1193897151529874e-06</v>
+        <v>-1.7823892669612852e-05</v>
       </c>
       <c r="S23">
-        <v>-2.1592972747274189e-05</v>
+        <v>-1.6540941160553139e-05</v>
       </c>
       <c r="T23">
-        <v>2.190562178820514e-05</v>
+        <v>9.8248452292374992e-05</v>
       </c>
       <c r="U23">
-        <v>2.8191657824618455e-05</v>
+        <v>9.1066052044852259e-05</v>
       </c>
       <c r="V23">
-        <v>2.2910447972973938e-05</v>
+        <v>5.8590977754004788e-05</v>
       </c>
       <c r="W23">
-        <v>0.00021111983175499925</v>
+        <v>0.00016636127862838999</v>
       </c>
       <c r="X23">
-        <v>0.00053996478025711053</v>
+        <v>0.00040067938195212241</v>
       </c>
       <c r="Y23">
-        <v>0.00022623288523965224</v>
+        <v>0.00017854780852958842</v>
       </c>
       <c r="Z23">
-        <v>1.0090656048973535e-05</v>
+        <v>-1.4819805628393432e-05</v>
       </c>
       <c r="AA23">
-        <v>1.5038794390850993e-05</v>
+        <v>-1.5540206249952911e-05</v>
       </c>
       <c r="AB23">
-        <v>2.395369186708842e-05</v>
+        <v>-1.5218837537113125e-06</v>
       </c>
       <c r="AC23">
-        <v>1.8834833522594766e-05</v>
+        <v>-6.7203803147305443e-06</v>
       </c>
       <c r="AD23">
-        <v>5.9793821400408779e-05</v>
+        <v>1.9219754684363105e-05</v>
       </c>
       <c r="AE23">
-        <v>1.1611884530182302e-05</v>
+        <v>-2.7750565127864939e-05</v>
       </c>
       <c r="AF23">
-        <v>-2.6925762539104889e-07</v>
+        <v>-7.6999422546614844e-07</v>
       </c>
       <c r="AG23">
-        <v>0.00011623267111935905</v>
+        <v>9.5602396610584188e-05</v>
       </c>
       <c r="AH23">
-        <v>1.5389163367935809e-05</v>
+        <v>7.974738377641258e-06</v>
       </c>
       <c r="AI23">
-        <v>-0.0012783098564462269</v>
+        <v>-0.00099830234275434309</v>
       </c>
     </row>
     <row r="24">
@@ -6799,106 +6799,106 @@
         <v>51</v>
       </c>
       <c r="B24">
-        <v>0.60155594803663481</v>
+        <v>0.21517368165845735</v>
       </c>
       <c r="C24">
-        <v>0.00013694080783844886</v>
+        <v>0.00010297790051462028</v>
       </c>
       <c r="D24">
-        <v>1.0265266595365681e-05</v>
+        <v>9.8901673089887138e-06</v>
       </c>
       <c r="E24">
-        <v>-1.8130713169339472e-08</v>
+        <v>-3.7547868734137601e-08</v>
       </c>
       <c r="F24">
-        <v>5.9715548943519012e-05</v>
+        <v>3.1718669050096599e-05</v>
       </c>
       <c r="G24">
-        <v>0.00011715946216607118</v>
+        <v>8.6282675976143792e-05</v>
       </c>
       <c r="H24">
-        <v>0.00014344774122373918</v>
+        <v>9.836435578030071e-05</v>
       </c>
       <c r="I24">
-        <v>0.00013852717240664609</v>
+        <v>0.00010371067588002786</v>
       </c>
       <c r="J24">
-        <v>-5.816469041652558e-05</v>
+        <v>-2.1306315218930899e-05</v>
       </c>
       <c r="K24">
-        <v>4.6191887562013366e-05</v>
+        <v>5.5120278635650984e-05</v>
       </c>
       <c r="L24">
-        <v>8.6033118555267458e-06</v>
+        <v>3.9968723023051736e-06</v>
       </c>
       <c r="M24">
-        <v>-0.00019737655532720032</v>
+        <v>-3.5140046851827511e-05</v>
       </c>
       <c r="N24">
-        <v>-0.00012331938187331941</v>
+        <v>-9.8619098376432311e-05</v>
       </c>
       <c r="O24">
-        <v>5.7313670718088842e-05</v>
+        <v>2.2703858386491338e-05</v>
       </c>
       <c r="P24">
-        <v>0.00016661892369636234</v>
+        <v>2.316996492159111e-05</v>
       </c>
       <c r="Q24">
-        <v>0.00023147393001431062</v>
+        <v>0.0001220726888068787</v>
       </c>
       <c r="R24">
-        <v>9.3570909470648382e-05</v>
+        <v>5.2840393465285705e-06</v>
       </c>
       <c r="S24">
-        <v>0.00021078688298528658</v>
+        <v>0.0001029112026425011</v>
       </c>
       <c r="T24">
-        <v>0.0007232136229608525</v>
+        <v>0.00070207492734455923</v>
       </c>
       <c r="U24">
-        <v>0.00051999392204682676</v>
+        <v>0.00057607957093675508</v>
       </c>
       <c r="V24">
-        <v>0.00049063200750470645</v>
+        <v>0.00053790788706125064</v>
       </c>
       <c r="W24">
-        <v>0.00032374727392850693</v>
+        <v>0.00025073862351095399</v>
       </c>
       <c r="X24">
-        <v>0.00022623288523965224</v>
+        <v>0.00017854780852958842</v>
       </c>
       <c r="Y24">
-        <v>0.0049391707950833235</v>
+        <v>0.0033872444461233967</v>
       </c>
       <c r="Z24">
-        <v>4.1001920201236318e-05</v>
+        <v>2.8285800909851966e-06</v>
       </c>
       <c r="AA24">
-        <v>5.8546293138214242e-05</v>
+        <v>2.6390516142182593e-05</v>
       </c>
       <c r="AB24">
-        <v>8.9294459759380824e-05</v>
+        <v>4.8858054046928959e-05</v>
       </c>
       <c r="AC24">
-        <v>3.0241719546356469e-05</v>
+        <v>-7.622718019915215e-07</v>
       </c>
       <c r="AD24">
-        <v>9.1352888362737433e-05</v>
+        <v>3.5780002498820378e-05</v>
       </c>
       <c r="AE24">
-        <v>-3.5884440126575035e-05</v>
+        <v>-7.4989240712913642e-05</v>
       </c>
       <c r="AF24">
-        <v>-8.8393577961908054e-06</v>
+        <v>-4.8846479974168429e-06</v>
       </c>
       <c r="AG24">
-        <v>6.0175165015133813e-05</v>
+        <v>2.1838411203416522e-05</v>
       </c>
       <c r="AH24">
-        <v>1.0711515924385082e-05</v>
+        <v>1.3512546714689229e-05</v>
       </c>
       <c r="AI24">
-        <v>-0.0011984065111760687</v>
+        <v>-0.001090271946000361</v>
       </c>
     </row>
     <row r="25">
@@ -6906,106 +6906,106 @@
         <v>52</v>
       </c>
       <c r="B25">
-        <v>-0.17667000773885255</v>
+        <v>-0.10278586913875591</v>
       </c>
       <c r="C25">
-        <v>5.7425833494780031e-06</v>
+        <v>-9.335864421748392e-06</v>
       </c>
       <c r="D25">
-        <v>-3.6890395435922214e-07</v>
+        <v>9.1350952081012903e-07</v>
       </c>
       <c r="E25">
-        <v>-5.5115163241112756e-09</v>
+        <v>-3.6069770294001315e-08</v>
       </c>
       <c r="F25">
-        <v>-5.6077131279566074e-05</v>
+        <v>-5.1834310924630395e-05</v>
       </c>
       <c r="G25">
-        <v>-3.2391368146266614e-05</v>
+        <v>-2.3694207330035404e-05</v>
       </c>
       <c r="H25">
-        <v>-7.1874354112027878e-05</v>
+        <v>-7.6247231313643794e-05</v>
       </c>
       <c r="I25">
-        <v>-6.0315393916438552e-06</v>
+        <v>1.1164296909034824e-05</v>
       </c>
       <c r="J25">
-        <v>8.5149803357657992e-06</v>
+        <v>7.2757498058676063e-06</v>
       </c>
       <c r="K25">
-        <v>9.418187349832124e-06</v>
+        <v>2.1383848145603915e-05</v>
       </c>
       <c r="L25">
-        <v>-5.8983953549960456e-06</v>
+        <v>-9.6109704479998775e-06</v>
       </c>
       <c r="M25">
-        <v>-5.2793343367700959e-05</v>
+        <v>-1.0553378979036472e-05</v>
       </c>
       <c r="N25">
-        <v>6.3892697498914601e-05</v>
+        <v>0.00012401814429304544</v>
       </c>
       <c r="O25">
-        <v>-0.00011547568708166747</v>
+        <v>-4.1741491435329258e-05</v>
       </c>
       <c r="P25">
-        <v>8.6525314375642546e-05</v>
+        <v>2.8500856413521142e-05</v>
       </c>
       <c r="Q25">
-        <v>-1.4248406050923479e-05</v>
+        <v>6.6182500210149042e-05</v>
       </c>
       <c r="R25">
-        <v>9.9286993257364023e-06</v>
+        <v>6.7856582924429899e-05</v>
       </c>
       <c r="S25">
-        <v>-1.6892185388245676e-05</v>
+        <v>1.5977289439899484e-05</v>
       </c>
       <c r="T25">
-        <v>-2.1245397239001707e-06</v>
+        <v>8.1796134884655827e-05</v>
       </c>
       <c r="U25">
-        <v>6.6557231107324325e-05</v>
+        <v>0.00018260500360920383</v>
       </c>
       <c r="V25">
-        <v>3.2379196705672499e-05</v>
+        <v>0.00020058416387127957</v>
       </c>
       <c r="W25">
-        <v>-2.8259794567796529e-07</v>
+        <v>1.1209677716053802e-05</v>
       </c>
       <c r="X25">
-        <v>1.0090656048973535e-05</v>
+        <v>-1.4819805628393432e-05</v>
       </c>
       <c r="Y25">
-        <v>4.1001920201236318e-05</v>
+        <v>2.8285800909851966e-06</v>
       </c>
       <c r="Z25">
-        <v>0.0027368841041138471</v>
+        <v>0.0023639021397631331</v>
       </c>
       <c r="AA25">
-        <v>0.002403550398369916</v>
+        <v>0.0021223492808096116</v>
       </c>
       <c r="AB25">
-        <v>0.0024018384466925175</v>
+        <v>0.0021256421183058131</v>
       </c>
       <c r="AC25">
-        <v>0.0024068293784165707</v>
+        <v>0.0021240227273291684</v>
       </c>
       <c r="AD25">
-        <v>0.0024144940450831001</v>
+        <v>0.0021274580204613961</v>
       </c>
       <c r="AE25">
-        <v>0.0023958525996362438</v>
+        <v>0.002109964130242789</v>
       </c>
       <c r="AF25">
-        <v>6.8893600317669401e-06</v>
+        <v>8.2309305574250539e-06</v>
       </c>
       <c r="AG25">
-        <v>3.8664036657134679e-05</v>
+        <v>4.8591971455376384e-05</v>
       </c>
       <c r="AH25">
-        <v>6.6604240827844267e-06</v>
+        <v>-2.6220638622332726e-05</v>
       </c>
       <c r="AI25">
-        <v>-0.0024100460320740777</v>
+        <v>-0.0023158348738640863</v>
       </c>
     </row>
     <row r="26">
@@ -7013,106 +7013,106 @@
         <v>53</v>
       </c>
       <c r="B26">
-        <v>-0.041384073498688286</v>
+        <v>-0.036225405680923375</v>
       </c>
       <c r="C26">
-        <v>1.0743021050413368e-05</v>
+        <v>-5.8546447618001047e-06</v>
       </c>
       <c r="D26">
-        <v>2.7230093151540838e-06</v>
+        <v>3.6215784504039074e-06</v>
       </c>
       <c r="E26">
-        <v>-4.0942454040429362e-08</v>
+        <v>-6.8712749839840212e-08</v>
       </c>
       <c r="F26">
-        <v>-3.2613800962478764e-05</v>
+        <v>-3.7256828155836277e-05</v>
       </c>
       <c r="G26">
-        <v>-3.342869865768038e-05</v>
+        <v>-2.6420656955067042e-05</v>
       </c>
       <c r="H26">
-        <v>-8.9556933801142932e-05</v>
+        <v>-9.1057264796521155e-05</v>
       </c>
       <c r="I26">
-        <v>-5.561515106820218e-05</v>
+        <v>-2.9495735676815082e-05</v>
       </c>
       <c r="J26">
-        <v>7.7232169495954248e-06</v>
+        <v>6.9017503300158681e-06</v>
       </c>
       <c r="K26">
-        <v>-1.9276415664130865e-05</v>
+        <v>4.0595445390421633e-06</v>
       </c>
       <c r="L26">
-        <v>-8.370704189693698e-06</v>
+        <v>-1.1695178700563376e-05</v>
       </c>
       <c r="M26">
-        <v>-8.174737975831258e-05</v>
+        <v>-1.5697155095718355e-05</v>
       </c>
       <c r="N26">
-        <v>0.00011439383984365313</v>
+        <v>0.00016044528123872084</v>
       </c>
       <c r="O26">
-        <v>-9.553782629575147e-05</v>
+        <v>-3.7558632074420238e-05</v>
       </c>
       <c r="P26">
-        <v>0.00010835578757822277</v>
+        <v>3.1628420065588504e-05</v>
       </c>
       <c r="Q26">
-        <v>4.6359194890806775e-05</v>
+        <v>9.487294352295006e-05</v>
       </c>
       <c r="R26">
-        <v>6.572844696292211e-05</v>
+        <v>0.00010159802617199822</v>
       </c>
       <c r="S26">
-        <v>4.3026856138298538e-05</v>
+        <v>4.9367833054357949e-05</v>
       </c>
       <c r="T26">
-        <v>-0.00023697175779435059</v>
+        <v>-6.5977748268545265e-05</v>
       </c>
       <c r="U26">
-        <v>-0.00015827837842209442</v>
+        <v>4.8086735575649138e-05</v>
       </c>
       <c r="V26">
-        <v>-0.00019517041910760771</v>
+        <v>7.8774566333253936e-05</v>
       </c>
       <c r="W26">
-        <v>-1.2850461832927804e-05</v>
+        <v>3.0164766362266756e-06</v>
       </c>
       <c r="X26">
-        <v>1.5038794390850993e-05</v>
+        <v>-1.5540206249952911e-05</v>
       </c>
       <c r="Y26">
-        <v>5.8546293138214242e-05</v>
+        <v>2.6390516142182593e-05</v>
       </c>
       <c r="Z26">
-        <v>0.002403550398369916</v>
+        <v>0.0021223492808096116</v>
       </c>
       <c r="AA26">
-        <v>0.0029148475551923816</v>
+        <v>0.0024772697194631902</v>
       </c>
       <c r="AB26">
-        <v>0.0024160957126365826</v>
+        <v>0.0021351677875133183</v>
       </c>
       <c r="AC26">
-        <v>0.0024093572699213821</v>
+        <v>0.002125110038320336</v>
       </c>
       <c r="AD26">
-        <v>0.0024199231391288829</v>
+        <v>0.0021300649491891146</v>
       </c>
       <c r="AE26">
-        <v>0.0023976319659872111</v>
+        <v>0.0021116197683530651</v>
       </c>
       <c r="AF26">
-        <v>5.039172834197763e-06</v>
+        <v>6.9238386467466201e-06</v>
       </c>
       <c r="AG26">
-        <v>3.4835930301661648e-05</v>
+        <v>5.7692432346097104e-05</v>
       </c>
       <c r="AH26">
-        <v>-2.8199243767408622e-05</v>
+        <v>-3.7669613783008625e-05</v>
       </c>
       <c r="AI26">
-        <v>-0.0022004278612251281</v>
+        <v>-0.0021911353971823654</v>
       </c>
     </row>
     <row r="27">
@@ -7120,106 +7120,106 @@
         <v>54</v>
       </c>
       <c r="B27">
-        <v>-0.041511225058046997</v>
+        <v>-0.051789723528653145</v>
       </c>
       <c r="C27">
-        <v>6.9760191377979161e-06</v>
+        <v>-1.0585656419178065e-05</v>
       </c>
       <c r="D27">
-        <v>2.6496366877957415e-06</v>
+        <v>4.3609333452371355e-06</v>
       </c>
       <c r="E27">
-        <v>-3.9895281830393476e-08</v>
+        <v>-7.3442178562350164e-08</v>
       </c>
       <c r="F27">
-        <v>-4.3719027208413697e-05</v>
+        <v>-4.3119877050201987e-05</v>
       </c>
       <c r="G27">
-        <v>-3.4709028774606351e-05</v>
+        <v>-2.4660131683162771e-05</v>
       </c>
       <c r="H27">
-        <v>-9.6477235923793717e-05</v>
+        <v>-9.1372038908214153e-05</v>
       </c>
       <c r="I27">
-        <v>-7.6338942696981579e-05</v>
+        <v>-4.0220255936107693e-05</v>
       </c>
       <c r="J27">
-        <v>-9.9065126713600744e-06</v>
+        <v>2.632259753434833e-06</v>
       </c>
       <c r="K27">
-        <v>-2.7012175418189175e-05</v>
+        <v>-2.5227767774379725e-06</v>
       </c>
       <c r="L27">
-        <v>-4.4093195581566065e-06</v>
+        <v>-8.7266002255603918e-06</v>
       </c>
       <c r="M27">
-        <v>-7.4798169395010197e-05</v>
+        <v>-1.7947351872157482e-05</v>
       </c>
       <c r="N27">
-        <v>0.00013461317724291501</v>
+        <v>0.00019725792838860698</v>
       </c>
       <c r="O27">
-        <v>-0.00010038128288236559</v>
+        <v>-3.7989180969422463e-05</v>
       </c>
       <c r="P27">
-        <v>8.8851153156342948e-05</v>
+        <v>3.4950511344949709e-05</v>
       </c>
       <c r="Q27">
-        <v>9.9282122083284253e-05</v>
+        <v>0.00015783475030169613</v>
       </c>
       <c r="R27">
-        <v>7.9839508586744285e-05</v>
+        <v>0.00013175722019482779</v>
       </c>
       <c r="S27">
-        <v>7.0954999775664626e-05</v>
+        <v>8.5799646120243581e-05</v>
       </c>
       <c r="T27">
-        <v>-0.00023627816261422669</v>
+        <v>-8.1554675259494763e-05</v>
       </c>
       <c r="U27">
-        <v>-0.00021599875091771149</v>
+        <v>-5.1239361966075401e-06</v>
       </c>
       <c r="V27">
-        <v>-0.0002307304293205051</v>
+        <v>3.6505203233518167e-05</v>
       </c>
       <c r="W27">
-        <v>8.9035697779476348e-07</v>
+        <v>1.6215172945386385e-05</v>
       </c>
       <c r="X27">
-        <v>2.395369186708842e-05</v>
+        <v>-1.5218837537113125e-06</v>
       </c>
       <c r="Y27">
-        <v>8.9294459759380824e-05</v>
+        <v>4.8858054046928959e-05</v>
       </c>
       <c r="Z27">
-        <v>0.0024018384466925175</v>
+        <v>0.0021256421183058131</v>
       </c>
       <c r="AA27">
-        <v>0.0024160957126365826</v>
+        <v>0.0021351677875133183</v>
       </c>
       <c r="AB27">
-        <v>0.0028912112699131546</v>
+        <v>0.0024572812342327803</v>
       </c>
       <c r="AC27">
-        <v>0.0024058644118620937</v>
+        <v>0.0021270935360720982</v>
       </c>
       <c r="AD27">
-        <v>0.0024182207010879434</v>
+        <v>0.0021350028532362876</v>
       </c>
       <c r="AE27">
-        <v>0.0023938239766845499</v>
+        <v>0.0021126325070296315</v>
       </c>
       <c r="AF27">
-        <v>3.9742914039158828e-06</v>
+        <v>6.3410570567871928e-06</v>
       </c>
       <c r="AG27">
-        <v>8.5101182829898977e-05</v>
+        <v>7.1950381959264009e-05</v>
       </c>
       <c r="AH27">
-        <v>1.9214496868034817e-05</v>
+        <v>-2.2614177046242478e-05</v>
       </c>
       <c r="AI27">
-        <v>-0.0021712246245258688</v>
+        <v>-0.0022047320839206708</v>
       </c>
     </row>
     <row r="28">
@@ -7227,106 +7227,106 @@
         <v>55</v>
       </c>
       <c r="B28">
-        <v>-0.17274750090494068</v>
+        <v>-0.10264379271074485</v>
       </c>
       <c r="C28">
-        <v>4.37177101838762e-06</v>
+        <v>-8.7572897623118122e-06</v>
       </c>
       <c r="D28">
-        <v>3.3060123068474884e-06</v>
+        <v>3.6727555877707108e-06</v>
       </c>
       <c r="E28">
-        <v>-4.6005625474448603e-08</v>
+        <v>-6.6999920756369802e-08</v>
       </c>
       <c r="F28">
-        <v>-9.434248749252863e-05</v>
+        <v>-7.7778989518010634e-05</v>
       </c>
       <c r="G28">
-        <v>-9.5431062887091789e-05</v>
+        <v>-7.3953676822698881e-05</v>
       </c>
       <c r="H28">
-        <v>-0.00014693418837219137</v>
+        <v>-0.00013429476518331436</v>
       </c>
       <c r="I28">
-        <v>-9.1646211952361393e-05</v>
+        <v>-5.789279880685479e-05</v>
       </c>
       <c r="J28">
-        <v>9.5318444476418823e-06</v>
+        <v>8.3152163847382398e-06</v>
       </c>
       <c r="K28">
-        <v>7.8577577430050637e-06</v>
+        <v>2.1739266659929926e-05</v>
       </c>
       <c r="L28">
-        <v>-7.1575627419663402e-06</v>
+        <v>-1.0450915284128772e-05</v>
       </c>
       <c r="M28">
-        <v>-6.6566042929599653e-05</v>
+        <v>-1.3303158559206591e-05</v>
       </c>
       <c r="N28">
-        <v>9.7898026577931821e-05</v>
+        <v>0.00014651550897268654</v>
       </c>
       <c r="O28">
-        <v>-0.00012848653550902875</v>
+        <v>-4.6037538605574115e-05</v>
       </c>
       <c r="P28">
-        <v>0.00010941218739209991</v>
+        <v>3.1764693548203232e-05</v>
       </c>
       <c r="Q28">
-        <v>-3.4653852526901445e-05</v>
+        <v>3.0762400758397104e-05</v>
       </c>
       <c r="R28">
-        <v>1.0444425434076934e-05</v>
+        <v>5.4821079419653182e-05</v>
       </c>
       <c r="S28">
-        <v>-6.8574665755454303e-06</v>
+        <v>6.352830463492512e-06</v>
       </c>
       <c r="T28">
-        <v>-4.9982022240475585e-05</v>
+        <v>5.5011388798308428e-05</v>
       </c>
       <c r="U28">
-        <v>5.6598753435136047e-05</v>
+        <v>0.00019026714922081717</v>
       </c>
       <c r="V28">
-        <v>5.0429980654251652e-05</v>
+        <v>0.00023111009227154682</v>
       </c>
       <c r="W28">
-        <v>-6.1956261635208589e-06</v>
+        <v>8.347343052448163e-06</v>
       </c>
       <c r="X28">
-        <v>1.8834833522594766e-05</v>
+        <v>-6.7203803147305443e-06</v>
       </c>
       <c r="Y28">
-        <v>3.0241719546356469e-05</v>
+        <v>-7.622718019915215e-07</v>
       </c>
       <c r="Z28">
-        <v>0.0024068293784165707</v>
+        <v>0.0021240227273291684</v>
       </c>
       <c r="AA28">
-        <v>0.0024093572699213821</v>
+        <v>0.002125110038320336</v>
       </c>
       <c r="AB28">
-        <v>0.0024058644118620937</v>
+        <v>0.0021270935360720982</v>
       </c>
       <c r="AC28">
-        <v>0.0027382482436391796</v>
+        <v>0.0023633643182878962</v>
       </c>
       <c r="AD28">
-        <v>0.0024168318782956813</v>
+        <v>0.0021270264141845779</v>
       </c>
       <c r="AE28">
-        <v>0.0024003266541567266</v>
+        <v>0.002112266810682553</v>
       </c>
       <c r="AF28">
-        <v>7.3384980026480068e-06</v>
+        <v>8.948103966095376e-06</v>
       </c>
       <c r="AG28">
-        <v>3.0650755195742868e-05</v>
+        <v>4.8606877753752144e-05</v>
       </c>
       <c r="AH28">
-        <v>-1.8159970944595571e-05</v>
+        <v>-5.2841160719077781e-05</v>
       </c>
       <c r="AI28">
-        <v>-0.0023882160995456758</v>
+        <v>-0.0023054847195037266</v>
       </c>
     </row>
     <row r="29">
@@ -7334,106 +7334,106 @@
         <v>56</v>
       </c>
       <c r="B29">
-        <v>-0.059646042206067167</v>
+        <v>-0.048350971377519043</v>
       </c>
       <c r="C29">
-        <v>-1.8893322566322499e-05</v>
+        <v>-2.4432389547118601e-05</v>
       </c>
       <c r="D29">
-        <v>2.7000313798056935e-06</v>
+        <v>3.6196768917586006e-06</v>
       </c>
       <c r="E29">
-        <v>-3.3621964339694341e-08</v>
+        <v>-6.1898072402069532e-08</v>
       </c>
       <c r="F29">
-        <v>1.0024030448895545e-05</v>
+        <v>-1.8384535306178919e-06</v>
       </c>
       <c r="G29">
-        <v>-4.4670324184873517e-07</v>
+        <v>-1.3619129778063492e-05</v>
       </c>
       <c r="H29">
-        <v>-5.8249228400782897e-05</v>
+        <v>-6.8257765771505079e-05</v>
       </c>
       <c r="I29">
-        <v>4.7353825128320683e-05</v>
+        <v>4.768166417012964e-05</v>
       </c>
       <c r="J29">
-        <v>-7.4128590388704578e-05</v>
+        <v>-9.1512358603782229e-06</v>
       </c>
       <c r="K29">
-        <v>-1.7723351807230679e-05</v>
+        <v>2.4285883841762448e-06</v>
       </c>
       <c r="L29">
-        <v>-1.0905681299324917e-05</v>
+        <v>-1.2277464137015223e-05</v>
       </c>
       <c r="M29">
-        <v>-5.2188146467307259e-05</v>
+        <v>-1.1053181640752294e-05</v>
       </c>
       <c r="N29">
-        <v>7.1443082540535198e-05</v>
+        <v>0.00012474930381014453</v>
       </c>
       <c r="O29">
-        <v>-4.7242070389820132e-05</v>
+        <v>-3.7540151969539556e-05</v>
       </c>
       <c r="P29">
-        <v>6.8524030885496129e-05</v>
+        <v>2.9113856266219703e-05</v>
       </c>
       <c r="Q29">
-        <v>6.5856619127423362e-05</v>
+        <v>0.00011287110516250659</v>
       </c>
       <c r="R29">
-        <v>8.7148450729574757e-05</v>
+        <v>0.00011607455231191243</v>
       </c>
       <c r="S29">
-        <v>5.9035760047622746e-05</v>
+        <v>5.9201836919625228e-05</v>
       </c>
       <c r="T29">
-        <v>-0.00029799213440012858</v>
+        <v>-0.00010304340954919852</v>
       </c>
       <c r="U29">
-        <v>-0.00021078048529140064</v>
+        <v>3.853106959384768e-07</v>
       </c>
       <c r="V29">
-        <v>-0.00023556963315815062</v>
+        <v>2.4134375351770807e-05</v>
       </c>
       <c r="W29">
-        <v>7.9580214339586058e-06</v>
+        <v>1.8218598874120664e-05</v>
       </c>
       <c r="X29">
-        <v>5.9793821400408779e-05</v>
+        <v>1.9219754684363105e-05</v>
       </c>
       <c r="Y29">
-        <v>9.1352888362737433e-05</v>
+        <v>3.5780002498820378e-05</v>
       </c>
       <c r="Z29">
-        <v>0.0024144940450831001</v>
+        <v>0.0021274580204613961</v>
       </c>
       <c r="AA29">
-        <v>0.0024199231391288829</v>
+        <v>0.0021300649491891146</v>
       </c>
       <c r="AB29">
-        <v>0.0024182207010879434</v>
+        <v>0.0021350028532362876</v>
       </c>
       <c r="AC29">
-        <v>0.0024168318782956813</v>
+        <v>0.0021270264141845779</v>
       </c>
       <c r="AD29">
-        <v>0.0027426640374758997</v>
+        <v>0.0023560558506151431</v>
       </c>
       <c r="AE29">
-        <v>0.0024013860735255625</v>
+        <v>0.0021110009035527756</v>
       </c>
       <c r="AF29">
-        <v>6.7317510321905603e-06</v>
+        <v>9.1173440295177805e-06</v>
       </c>
       <c r="AG29">
-        <v>0.00024879189554570264</v>
+        <v>0.00020040793013192601</v>
       </c>
       <c r="AH29">
-        <v>5.4293743339964631e-08</v>
+        <v>-3.24299948368668e-05</v>
       </c>
       <c r="AI29">
-        <v>-0.0022567947157818703</v>
+        <v>-0.0022442484931118984</v>
       </c>
     </row>
     <row r="30">
@@ -7441,106 +7441,106 @@
         <v>57</v>
       </c>
       <c r="B30">
-        <v>-0.15083426778561873</v>
+        <v>-0.11049107609094856</v>
       </c>
       <c r="C30">
-        <v>9.078395632183029e-06</v>
+        <v>-4.4127055464639188e-06</v>
       </c>
       <c r="D30">
-        <v>-3.7432941115907417e-06</v>
+        <v>-4.014368705582283e-06</v>
       </c>
       <c r="E30">
-        <v>1.8196754478072829e-08</v>
+        <v>-8.3402859556666785e-10</v>
       </c>
       <c r="F30">
-        <v>-5.3170062463804915e-06</v>
+        <v>-1.8419200261227565e-05</v>
       </c>
       <c r="G30">
-        <v>1.5892475574857154e-06</v>
+        <v>-4.6261090988816548e-06</v>
       </c>
       <c r="H30">
-        <v>-4.207361399925628e-05</v>
+        <v>-4.7055995359580351e-05</v>
       </c>
       <c r="I30">
-        <v>-1.1162008556380321e-05</v>
+        <v>6.7545297397632689e-06</v>
       </c>
       <c r="J30">
-        <v>-3.4362991330363968e-06</v>
+        <v>8.0240392261744832e-06</v>
       </c>
       <c r="K30">
-        <v>1.1960281701943796e-05</v>
+        <v>1.3038864400544787e-05</v>
       </c>
       <c r="L30">
-        <v>-5.2561162497527967e-06</v>
+        <v>-9.1444009299757552e-06</v>
       </c>
       <c r="M30">
-        <v>-5.4707719815161954e-05</v>
+        <v>-1.2242476380704357e-05</v>
       </c>
       <c r="N30">
-        <v>0.00012350157466021208</v>
+        <v>0.0001852813442095532</v>
       </c>
       <c r="O30">
-        <v>-9.497152143127203e-05</v>
+        <v>-4.3420541572997698e-05</v>
       </c>
       <c r="P30">
-        <v>5.8228554816225743e-05</v>
+        <v>2.6371509084704827e-05</v>
       </c>
       <c r="Q30">
-        <v>-4.8637700066664173e-07</v>
+        <v>7.3446356314997813e-05</v>
       </c>
       <c r="R30">
-        <v>3.6249155061806844e-05</v>
+        <v>9.5597050472739378e-05</v>
       </c>
       <c r="S30">
-        <v>1.7587982876780405e-05</v>
+        <v>4.3467628110373442e-05</v>
       </c>
       <c r="T30">
-        <v>-6.9971695066448243e-05</v>
+        <v>-8.9685666702423459e-05</v>
       </c>
       <c r="U30">
-        <v>6.7585007183653626e-05</v>
+        <v>9.3167404871446384e-05</v>
       </c>
       <c r="V30">
-        <v>5.9506652066179883e-05</v>
+        <v>0.0001348805627858201</v>
       </c>
       <c r="W30">
-        <v>-5.1787848250889523e-05</v>
+        <v>-4.794041635996373e-05</v>
       </c>
       <c r="X30">
-        <v>1.1611884530182302e-05</v>
+        <v>-2.7750565127864939e-05</v>
       </c>
       <c r="Y30">
-        <v>-3.5884440126575035e-05</v>
+        <v>-7.4989240712913642e-05</v>
       </c>
       <c r="Z30">
-        <v>0.0023958525996362438</v>
+        <v>0.002109964130242789</v>
       </c>
       <c r="AA30">
-        <v>0.0023976319659872111</v>
+        <v>0.0021116197683530651</v>
       </c>
       <c r="AB30">
-        <v>0.0023938239766845499</v>
+        <v>0.0021126325070296315</v>
       </c>
       <c r="AC30">
-        <v>0.0024003266541567266</v>
+        <v>0.002112266810682553</v>
       </c>
       <c r="AD30">
-        <v>0.0024013860735255625</v>
+        <v>0.0021110009035527756</v>
       </c>
       <c r="AE30">
-        <v>0.0028600629481484534</v>
+        <v>0.0024564957981944922</v>
       </c>
       <c r="AF30">
-        <v>4.6628558613332784e-06</v>
+        <v>5.8879662373217137e-06</v>
       </c>
       <c r="AG30">
-        <v>2.6252214162212316e-05</v>
+        <v>3.7142461486385121e-05</v>
       </c>
       <c r="AH30">
-        <v>-3.8857779376191403e-05</v>
+        <v>-6.7257423107632409e-05</v>
       </c>
       <c r="AI30">
-        <v>-0.0022968007437127974</v>
+        <v>-0.0020547465710433234</v>
       </c>
     </row>
     <row r="31">
@@ -7548,106 +7548,106 @@
         <v>58</v>
       </c>
       <c r="B31">
-        <v>0.022661376593080655</v>
+        <v>0.012156935219847684</v>
       </c>
       <c r="C31">
-        <v>-1.1713617503157034e-07</v>
+        <v>-1.3817237429177379e-07</v>
       </c>
       <c r="D31">
-        <v>-1.1073115482207998e-07</v>
+        <v>-1.3660476020046644e-07</v>
       </c>
       <c r="E31">
-        <v>-7.6469376919826121e-10</v>
+        <v>-9.5757793863241551e-11</v>
       </c>
       <c r="F31">
-        <v>-2.1296604221588067e-06</v>
+        <v>-1.2536112130698041e-07</v>
       </c>
       <c r="G31">
-        <v>-4.9904075742537298e-06</v>
+        <v>-2.8987659844247721e-06</v>
       </c>
       <c r="H31">
-        <v>-3.8069441577882174e-06</v>
+        <v>-2.1202340239441037e-06</v>
       </c>
       <c r="I31">
-        <v>-1.5413697275998045e-06</v>
+        <v>-2.5183170442093184e-07</v>
       </c>
       <c r="J31">
-        <v>-1.2655894037201618e-06</v>
+        <v>-6.6831626087156612e-07</v>
       </c>
       <c r="K31">
-        <v>8.2590497641914012e-07</v>
+        <v>8.397996004587753e-07</v>
       </c>
       <c r="L31">
-        <v>-2.708817252856624e-07</v>
+        <v>-1.7756947047362303e-07</v>
       </c>
       <c r="M31">
-        <v>4.5140438765156904e-06</v>
+        <v>1.1087454115216786e-06</v>
       </c>
       <c r="N31">
-        <v>-1.6835123396858036e-06</v>
+        <v>-5.421617844185672e-07</v>
       </c>
       <c r="O31">
-        <v>-2.9833865790864454e-06</v>
+        <v>-7.1055333476091166e-07</v>
       </c>
       <c r="P31">
-        <v>-4.835728867982459e-06</v>
+        <v>-1.0920358114035344e-06</v>
       </c>
       <c r="Q31">
-        <v>-4.2407887498384193e-06</v>
+        <v>-4.8402692097325375e-07</v>
       </c>
       <c r="R31">
-        <v>-8.6701134686602592e-06</v>
+        <v>-3.8478896559055505e-06</v>
       </c>
       <c r="S31">
-        <v>-1.1447210369927276e-05</v>
+        <v>-6.1333967309722153e-06</v>
       </c>
       <c r="T31">
-        <v>2.1528153876205439e-07</v>
+        <v>2.9647257412071418e-06</v>
       </c>
       <c r="U31">
-        <v>6.9688415398830176e-06</v>
+        <v>7.4139764138646432e-06</v>
       </c>
       <c r="V31">
-        <v>7.0868702618841553e-06</v>
+        <v>7.1148461006115976e-06</v>
       </c>
       <c r="W31">
-        <v>-1.6556312024076805e-08</v>
+        <v>-3.8638261772101368e-07</v>
       </c>
       <c r="X31">
-        <v>-2.6925762539104889e-07</v>
+        <v>-7.6999422546614844e-07</v>
       </c>
       <c r="Y31">
-        <v>-8.8393577961908054e-06</v>
+        <v>-4.8846479974168429e-06</v>
       </c>
       <c r="Z31">
-        <v>6.8893600317669401e-06</v>
+        <v>8.2309305574250539e-06</v>
       </c>
       <c r="AA31">
-        <v>5.039172834197763e-06</v>
+        <v>6.9238386467466201e-06</v>
       </c>
       <c r="AB31">
-        <v>3.9742914039158828e-06</v>
+        <v>6.3410570567871928e-06</v>
       </c>
       <c r="AC31">
-        <v>7.3384980026480068e-06</v>
+        <v>8.948103966095376e-06</v>
       </c>
       <c r="AD31">
-        <v>6.7317510321905603e-06</v>
+        <v>9.1173440295177805e-06</v>
       </c>
       <c r="AE31">
-        <v>4.6628558613332784e-06</v>
+        <v>5.8879662373217137e-06</v>
       </c>
       <c r="AF31">
-        <v>3.8250915107269126e-06</v>
+        <v>2.8421139156941524e-06</v>
       </c>
       <c r="AG31">
-        <v>-6.0227971973546426e-06</v>
+        <v>-4.1980285272648089e-06</v>
       </c>
       <c r="AH31">
-        <v>-1.1946887292048473e-05</v>
+        <v>-9.9133810261697846e-06</v>
       </c>
       <c r="AI31">
-        <v>-6.1465698923922151e-05</v>
+        <v>-5.0810842566947293e-05</v>
       </c>
     </row>
     <row r="32">
@@ -7655,106 +7655,106 @@
         <v>59</v>
       </c>
       <c r="B32">
-        <v>-0.20132120976842946</v>
+        <v>-0.16834303349841773</v>
       </c>
       <c r="C32">
-        <v>-7.8348589206558112e-05</v>
+        <v>-4.6110191547671093e-05</v>
       </c>
       <c r="D32">
-        <v>7.2371231071046956e-07</v>
+        <v>1.1014417681391481e-06</v>
       </c>
       <c r="E32">
-        <v>-2.1061352079788054e-08</v>
+        <v>-2.3560282270735233e-08</v>
       </c>
       <c r="F32">
-        <v>1.3101660560370029e-05</v>
+        <v>-1.6968138335860146e-05</v>
       </c>
       <c r="G32">
-        <v>2.3560435616849611e-05</v>
+        <v>2.3488971895614663e-06</v>
       </c>
       <c r="H32">
-        <v>-1.3115123110637311e-06</v>
+        <v>-2.752301032101466e-05</v>
       </c>
       <c r="I32">
-        <v>0.00017685683753167463</v>
+        <v>9.3093959670792308e-05</v>
       </c>
       <c r="J32">
-        <v>-0.00016898574867744656</v>
+        <v>-3.0264472768573137e-05</v>
       </c>
       <c r="K32">
-        <v>1.6152553236027049e-05</v>
+        <v>8.9231783656214085e-06</v>
       </c>
       <c r="L32">
-        <v>-5.157916866126524e-06</v>
+        <v>2.7865441998081248e-06</v>
       </c>
       <c r="M32">
-        <v>7.9398350037771e-05</v>
+        <v>1.290950570694912e-05</v>
       </c>
       <c r="N32">
-        <v>6.7252230678467063e-05</v>
+        <v>3.2833001582458464e-05</v>
       </c>
       <c r="O32">
-        <v>0.00017536319512749359</v>
+        <v>2.9504140180518852e-05</v>
       </c>
       <c r="P32">
-        <v>-4.5397950292241571e-05</v>
+        <v>-5.9418637690063832e-06</v>
       </c>
       <c r="Q32">
-        <v>0.00031659723868952827</v>
+        <v>0.00019026094556276463</v>
       </c>
       <c r="R32">
-        <v>0.0002879989900816636</v>
+        <v>0.00016438269767595284</v>
       </c>
       <c r="S32">
-        <v>0.0002006316169769623</v>
+        <v>0.0001026237763215327</v>
       </c>
       <c r="T32">
-        <v>-5.5994886211566119e-05</v>
+        <v>-6.2888099250091312e-06</v>
       </c>
       <c r="U32">
-        <v>2.6878304278842719e-05</v>
+        <v>7.9994971644315252e-05</v>
       </c>
       <c r="V32">
-        <v>9.5301536831786382e-05</v>
+        <v>0.00010872160819264814</v>
       </c>
       <c r="W32">
-        <v>3.3973305414521386e-05</v>
+        <v>3.4010345848732202e-05</v>
       </c>
       <c r="X32">
-        <v>0.00011623267111935905</v>
+        <v>9.5602396610584188e-05</v>
       </c>
       <c r="Y32">
-        <v>6.0175165015133813e-05</v>
+        <v>2.1838411203416522e-05</v>
       </c>
       <c r="Z32">
-        <v>3.8664036657134679e-05</v>
+        <v>4.8591971455376384e-05</v>
       </c>
       <c r="AA32">
-        <v>3.4835930301661648e-05</v>
+        <v>5.7692432346097104e-05</v>
       </c>
       <c r="AB32">
-        <v>8.5101182829898977e-05</v>
+        <v>7.1950381959264009e-05</v>
       </c>
       <c r="AC32">
-        <v>3.0650755195742868e-05</v>
+        <v>4.8606877753752144e-05</v>
       </c>
       <c r="AD32">
-        <v>0.00024879189554570264</v>
+        <v>0.00020040793013192601</v>
       </c>
       <c r="AE32">
-        <v>2.6252214162212316e-05</v>
+        <v>3.7142461486385121e-05</v>
       </c>
       <c r="AF32">
-        <v>-6.0227971973546426e-06</v>
+        <v>-4.1980285272648089e-06</v>
       </c>
       <c r="AG32">
-        <v>0.0017412523813394669</v>
+        <v>0.001308767589036399</v>
       </c>
       <c r="AH32">
-        <v>0.00028408191679715956</v>
+        <v>0.00014955068993683282</v>
       </c>
       <c r="AI32">
-        <v>-0.00031052205956822116</v>
+        <v>-0.0002592194314152793</v>
       </c>
     </row>
     <row r="33">
@@ -7762,106 +7762,106 @@
         <v>60</v>
       </c>
       <c r="B33">
-        <v>-0.12610477213348631</v>
+        <v>-0.14606536816231794</v>
       </c>
       <c r="C33">
-        <v>-2.871086252514396e-05</v>
+        <v>-1.7785141546052447e-05</v>
       </c>
       <c r="D33">
-        <v>-2.0665980981459645e-06</v>
+        <v>-1.6190327647853096e-07</v>
       </c>
       <c r="E33">
-        <v>9.6154898530007683e-09</v>
+        <v>-9.8789553017018076e-09</v>
       </c>
       <c r="F33">
-        <v>-1.1459651114999712e-06</v>
+        <v>-3.163277299217046e-06</v>
       </c>
       <c r="G33">
-        <v>5.04504162779848e-05</v>
+        <v>5.6548310784992374e-05</v>
       </c>
       <c r="H33">
-        <v>1.1186649182695282e-05</v>
+        <v>6.1610761025077295e-06</v>
       </c>
       <c r="I33">
-        <v>6.4684847934265953e-05</v>
+        <v>3.5675842478548499e-05</v>
       </c>
       <c r="J33">
-        <v>-8.3200465864430545e-05</v>
+        <v>-2.1851970220350368e-05</v>
       </c>
       <c r="K33">
-        <v>3.0176125816626896e-05</v>
+        <v>9.3125405626924085e-06</v>
       </c>
       <c r="L33">
-        <v>-7.1369518895646625e-06</v>
+        <v>-4.8713737517581206e-06</v>
       </c>
       <c r="M33">
-        <v>5.0290009126370559e-05</v>
+        <v>1.3523503522019133e-05</v>
       </c>
       <c r="N33">
-        <v>3.4368224754767647e-05</v>
+        <v>2.8941215185435436e-05</v>
       </c>
       <c r="O33">
-        <v>0.00022196014127580637</v>
+        <v>3.4805187773936431e-05</v>
       </c>
       <c r="P33">
-        <v>-0.00015119055836303815</v>
+        <v>-2.8616771146732921e-05</v>
       </c>
       <c r="Q33">
-        <v>0.00019594872205736056</v>
+        <v>9.7376897196153021e-05</v>
       </c>
       <c r="R33">
-        <v>0.0001867011565983975</v>
+        <v>9.4695687023475111e-05</v>
       </c>
       <c r="S33">
-        <v>0.00014512875049894208</v>
+        <v>7.1503295263667353e-05</v>
       </c>
       <c r="T33">
-        <v>0.00014858609909701621</v>
+        <v>1.4120930301418644e-05</v>
       </c>
       <c r="U33">
-        <v>0.00015217774312469186</v>
+        <v>1.3543670851434708e-05</v>
       </c>
       <c r="V33">
-        <v>0.00019727308075736388</v>
+        <v>7.3259343357217656e-05</v>
       </c>
       <c r="W33">
-        <v>-1.182606046036495e-05</v>
+        <v>-1.6129807065460138e-05</v>
       </c>
       <c r="X33">
-        <v>1.5389163367935809e-05</v>
+        <v>7.974738377641258e-06</v>
       </c>
       <c r="Y33">
-        <v>1.0711515924385082e-05</v>
+        <v>1.3512546714689229e-05</v>
       </c>
       <c r="Z33">
-        <v>6.6604240827844267e-06</v>
+        <v>-2.6220638622332726e-05</v>
       </c>
       <c r="AA33">
-        <v>-2.8199243767408622e-05</v>
+        <v>-3.7669613783008625e-05</v>
       </c>
       <c r="AB33">
-        <v>1.9214496868034817e-05</v>
+        <v>-2.2614177046242478e-05</v>
       </c>
       <c r="AC33">
-        <v>-1.8159970944595571e-05</v>
+        <v>-5.2841160719077781e-05</v>
       </c>
       <c r="AD33">
-        <v>5.4293743339964631e-08</v>
+        <v>-3.24299948368668e-05</v>
       </c>
       <c r="AE33">
-        <v>-3.8857779376191403e-05</v>
+        <v>-6.7257423107632409e-05</v>
       </c>
       <c r="AF33">
-        <v>-1.1946887292048473e-05</v>
+        <v>-9.9133810261697846e-06</v>
       </c>
       <c r="AG33">
-        <v>0.00028408191679715956</v>
+        <v>0.00014955068993683282</v>
       </c>
       <c r="AH33">
-        <v>0.0014618430071155078</v>
+        <v>0.0012169340638983968</v>
       </c>
       <c r="AI33">
-        <v>-0.00010223603091888482</v>
+        <v>8.9426217182326411e-05</v>
       </c>
     </row>
     <row r="34">
@@ -7869,106 +7869,106 @@
         <v>61</v>
       </c>
       <c r="B34">
-        <v>-0.44886908162203287</v>
+        <v>-0.31728577352928866</v>
       </c>
       <c r="C34">
-        <v>0.00017048838167084109</v>
+        <v>0.00015577358027267209</v>
       </c>
       <c r="D34">
-        <v>-0.00037840922310119454</v>
+        <v>-0.00027957227949393528</v>
       </c>
       <c r="E34">
-        <v>3.2688604033339336e-06</v>
+        <v>2.4101841408793162e-06</v>
       </c>
       <c r="F34">
-        <v>-0.0031907660066190684</v>
+        <v>-0.0024347903066560409</v>
       </c>
       <c r="G34">
-        <v>-0.003264930078864586</v>
+        <v>-0.0025068716653706587</v>
       </c>
       <c r="H34">
-        <v>-0.0033820336201729473</v>
+        <v>-0.0024907840804877122</v>
       </c>
       <c r="I34">
-        <v>-0.0039016022318896365</v>
+        <v>-0.0029982245594123175</v>
       </c>
       <c r="J34">
-        <v>0.00037411143719150966</v>
+        <v>8.019374920288896e-05</v>
       </c>
       <c r="K34">
-        <v>-0.0024598768867113464</v>
+        <v>-0.00187831800198429</v>
       </c>
       <c r="L34">
-        <v>8.0841463138480685e-05</v>
+        <v>7.2341622901808439e-05</v>
       </c>
       <c r="M34">
-        <v>-0.00010912148249779828</v>
+        <v>-1.905461139721737e-05</v>
       </c>
       <c r="N34">
-        <v>-0.0044423224796542029</v>
+        <v>-0.003199411113164013</v>
       </c>
       <c r="O34">
-        <v>-0.0037023871339994029</v>
+        <v>-0.00066844723513465412</v>
       </c>
       <c r="P34">
-        <v>-0.0031849625751416287</v>
+        <v>-0.00097849154912832176</v>
       </c>
       <c r="Q34">
-        <v>-0.015825749025517082</v>
+        <v>-0.011551297423127107</v>
       </c>
       <c r="R34">
-        <v>-0.01502158810750011</v>
+        <v>-0.0108666916165113</v>
       </c>
       <c r="S34">
-        <v>-0.014763368816508946</v>
+        <v>-0.010715118799295528</v>
       </c>
       <c r="T34">
-        <v>-0.024416804220154135</v>
+        <v>-0.018831810835430202</v>
       </c>
       <c r="U34">
-        <v>-0.019556821768951863</v>
+        <v>-0.014929297964842797</v>
       </c>
       <c r="V34">
-        <v>-0.019970339422381342</v>
+        <v>-0.015225895337582101</v>
       </c>
       <c r="W34">
-        <v>-0.00042718926414069328</v>
+        <v>-0.00041631372711569385</v>
       </c>
       <c r="X34">
-        <v>-0.0012783098564462269</v>
+        <v>-0.00099830234275434309</v>
       </c>
       <c r="Y34">
-        <v>-0.0011984065111760687</v>
+        <v>-0.001090271946000361</v>
       </c>
       <c r="Z34">
-        <v>-0.0024100460320740777</v>
+        <v>-0.0023158348738640863</v>
       </c>
       <c r="AA34">
-        <v>-0.0022004278612251281</v>
+        <v>-0.0021911353971823654</v>
       </c>
       <c r="AB34">
-        <v>-0.0021712246245258688</v>
+        <v>-0.0022047320839206708</v>
       </c>
       <c r="AC34">
-        <v>-0.0023882160995456758</v>
+        <v>-0.0023054847195037266</v>
       </c>
       <c r="AD34">
-        <v>-0.0022567947157818703</v>
+        <v>-0.0022442484931118984</v>
       </c>
       <c r="AE34">
-        <v>-0.0022968007437127974</v>
+        <v>-0.0020547465710433234</v>
       </c>
       <c r="AF34">
-        <v>-6.1465698923922151e-05</v>
+        <v>-5.0810842566947293e-05</v>
       </c>
       <c r="AG34">
-        <v>-0.00031052205956822116</v>
+        <v>-0.0002592194314152793</v>
       </c>
       <c r="AH34">
-        <v>-0.00010223603091888482</v>
+        <v>8.9426217182326411e-05</v>
       </c>
       <c r="AI34">
-        <v>0.051766342372952509</v>
+        <v>0.039259369291388263</v>
       </c>
     </row>
   </sheetData>

</xml_diff>